<commit_message>
Expand story branches and configured art pools
</commit_message>
<xml_diff>
--- a/story-config.xlsx
+++ b/story-config.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Choices" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StatusLines" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ArtPools" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -436,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -472,9 +473,9 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>雷劫散后，西陵旧议厅的水镜忽然亮起。天机营把铜门裂纹拓在镜中，冰心堂带来城外疫民名单，魍魉长老只问一句：上一世，是谁把这道裂纹藏起来的？
+          <t>雷劫散后，西陵旧议厅的水镜亮起。天机营、冰心堂、魍魉、云麓、荒火都派人入席，却没有一个人愿意先说真话。
 {{status}}
-这一幕的关键不再是“去哪”，而是你要先处理哪一个真实冲突。</t>
+你这一世不必急着选正邪，而要先决定从哪里撬开大荒的第一道缝。</t>
         </is>
       </c>
     </row>
@@ -489,9 +490,9 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>你已把第一条线索摆上桌面。遗墨的机关鸟落在梁上，吐出一片带盐痕的天书残页；冷喣没有看残页，只看你腰间的天命碎片。
+          <t>第一条线索已经落地，却把更多旧债牵了出来：铜门裂纹、城外疫民、北溟盐晶、沉船兵器、九天祭席，全都不像偶然。
 {{status}}
-现在故事开始分岔：公开残页会迫使诸门站队，私查北溟会更接近幽都旧约，强入铜门则可能让心魔提前醒来。</t>
+此时的选择会决定谁愿意信你，也会决定谁开始怕你。</t>
         </is>
       </c>
     </row>
@@ -501,14 +502,14 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>铜门显影</t>
+          <t>北溟旧约</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>铜门裂纹终于回应了你。水镜里先是北溟雪，再是东海神域的潮声，最后映出九天登神大典上一排没有名字的祭席。
+          <t>你沿着线索抵达北溟边境。雪原下埋着幽都旧约，海风里带着东海神域的潮声；某些神明把人间叫作试炼，也把牺牲叫作秩序。
 {{status}}
-这一幕已经接近终局。你可以补齐真相，也可以直接用修为撕开天门；若因果继续压上来，幽都会先替你作答。</t>
+真相变得更大，也更危险。你可以公开、潜入、修行、救人，或把自己推到铜门前。</t>
         </is>
       </c>
     </row>
@@ -518,13 +519,30 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
+          <t>东海神域</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>东海神域并非天外净土。潮宫残碑上写着九天与幽都的旧盟，神使说轮回是补天之器，魍魉影主却说那只是好听的锁链。
+{{status}}
+这一幕会把你的修炼方式变成结局倾向：守护者、破局者、独行者，或被因果拖入幽都。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
           <t>天命收束</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>本世的线索已经收束：诸门的旧账、幽都的误读、铜门的裂纹、九天的祭席，都指向同一个问题。
-力量足够时，你可以登九天；碎片足够时，你可以重订绝地天通；若因果压过道心，幽都会把你送回人间重走。</t>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>本世所有线索收束在铜门之前：诸门新约、幽都旧契、东海神域、九天祭席，都等你给出最后答案。
+道德越高，飞升越稳；因果越重，越容易先入幽都重走人间。正邪不是罪名，选择如何使用力量才是。</t>
         </is>
       </c>
     </row>
@@ -539,18 +557,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="56" customWidth="1" min="9" max="9"/>
+    <col width="62" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -633,7 +651,7 @@
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>魍魉席后一阵沉默。有人终于承认，铜门裂纹不是第一次出现。</t>
+          <t>魍魉席后一阵沉默。有人承认，铜门裂纹不是第一次出现。</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
@@ -708,14 +726,14 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>公开天书残页，迫诸门当场站队</t>
+          <t>借天机营兵符封锁铜门，逼各派留下证词</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -723,63 +741,71 @@
           <t>greatCouncil</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>karmaMax=35</t>
+        </is>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>virtue=8;karma=3</t>
+          <t>virtue=6;karma=6;fragments=1</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>诸门终于不再谈风骨，只开始谈各自欠下的债。</t>
+          <t>封锁不是仁慈，却让三个说谎的人同时露怯。</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>夜入北溟，追玄晶留下的幽都旧约</t>
+          <t>听云麓弟子推演星图，查裂纹对应的天象</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>northSea</t>
+          <t>tribulation</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>fragments=1;years=-1</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
+          <t>qi=18;years=-1</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>北溟风雪里，你听见幽都并不承认自己是地狱。</t>
+          <t>星图尽头不是九天，而是一片被抹去名字的海。</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>独自贴近铜门，听清门内喊出的名字</t>
+          <t>去荒火营查沉船兵器，不问来路先问用途</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -790,248 +816,268 @@
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>qi=16;karma=8</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
+          <t>qi=22;karma=6;years=-1</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
       <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>铜门没有打开，只把你的倒影换成了上一世的样子。</t>
+          <t>沉船铁锈里藏着神域火纹，像是专为破门而铸。</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>入镜阵审问心魔，先定自己的底线</t>
+          <t>不入议厅，先跟踪夜哭里的影步残象</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>heartDemon</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>karmaMin=20</t>
-        </is>
-      </c>
+          <t>foxRoad</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>memory=1</t>
+          <t>memory=1;karma=3</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
       <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>心魔没有退散，只把最锋利的问题留给你。</t>
+          <t>影步尽头留着半句誓词：救人者也会成为钥匙。</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>闭关冲境，用金丹火推开九天门缝</t>
+          <t>公开天书残页，迫诸门当场站队</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>tribulation</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>realmMax=4</t>
-        </is>
-      </c>
+          <t>greatCouncil</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>qi=34;years=-2</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
+          <t>virtue=8;karma=3</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>你把残页、药账、裂纹一并压入丹田，雷云再次聚拢。</t>
+          <t>诸门终于不再谈风骨，只开始谈各自欠下的债。</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B10" s="2" t="n">
-        <v>3</v>
-      </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>以碎片拼合旧约，提前重订绝地天通</t>
+          <t>夜入北溟，追玄晶留下的幽都旧约</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>breakWheel</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>fragmentsMin=4;realmMin=3</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr"/>
+          <t>northSea</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>fragments=1;years=-1</t>
+        </is>
+      </c>
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>北溟风雪里，你听见幽都并不承认自己是地狱。</t>
+        </is>
+      </c>
       <c r="J10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>登九天，直接问神明旧账</t>
+          <t>独自贴近铜门，听清门内喊出的名字</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>ascend</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>realmMin=5</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
+          <t>copperGate</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>qi=16;karma=8</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>铜门没有打开，只把你的倒影换成了上一世的样子。</t>
+        </is>
+      </c>
       <c r="J11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>以诸门新约重封铜门</t>
+          <t>请冰心堂先验疫民魂灯，查谁动过生死簿</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>breakWheel</t>
+          <t>iceHeart</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>fragmentsMin=4;virtueMin=60</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr"/>
+          <t>virtueMin=55</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>virtue=14;fragments=1;years=-1</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="inlineStr"/>
       <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>魂灯没有灭，说明有人把活人提前写进了死册。</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>登九天，看清祭席后的名字</t>
+          <t>与弈剑旧友论剑三夜，换他带你进旧阵眼</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>ascend</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>realmMin=5</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
+          <t>tribulation</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>qi=24;years=-2</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
       <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>剑意洗去浮躁，也削开阵眼外层的伪装。</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>因果压身，先入幽都照见本心</t>
+          <t>让魍魉暗网散出假消息，引蛇出洞</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>hell</t>
+          <t>shadow</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>karmaMin=55</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr"/>
+          <t>karmaMax=45</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>karma=9;fragments=1</t>
+        </is>
+      </c>
       <c r="G14" s="2" t="inlineStr"/>
       <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>这不是作恶，是用影子照出更深的影子。</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>寿元将尽，把本世线索交给下一世</t>
+          <t>护送一队凡人离开裂隙，暂缓追查</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1039,12 +1085,808 @@
           <t>death</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr"/>
-      <c r="F15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>yearsMin=1;virtueMin=80</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>virtue=18;memory=1;years=-1</t>
+        </is>
+      </c>
       <c r="G15" s="2" t="inlineStr"/>
       <c r="H15" s="2" t="inlineStr"/>
-      <c r="I15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>他们不知道真相，却会在下一世替你记得一个名字。</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>把北溟旧约带回议厅，要求诸门共证</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>greatCouncil</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>fragmentsMin=2</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>virtue=10;karma=5</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>旧约一出，最先拔剑的不是魔修，而是仙盟使者。</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>潜入幽都边市，查轮回簿被谁改写</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>hell</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>karmaMin=45</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>memory=2;karma=-8</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>幽都没有审你，只让你看见自己每次逃避的代价。</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>闭关炼化盐晶，冲击更高境界</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>tribulation</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>qi=38;years=-2</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>盐晶化作潮声，丹田里第一次出现神域门影。</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>救北溟雪灾里的敌派弟子，不问立场</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>iceHeart</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>virtue=20;karma=-6;years=-1</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>对方醒来后只说一句：原来你不是为了赢。</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>借荒火战阵强行撬开铜门外环</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>copperGate</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>realmMin=2</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>qi=30;karma=12;fragments=1;years=-2</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>铜门震动，九天祭席上有一个无名位被点亮。</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>用魍魉影契换取神域使者真名</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>heartDemon</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>karmaMin=20</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>fragments=1;karma=10;memory=1</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>你得到了真名，也听见心魔学会了那人的声音。</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>请太虚观召灵问古，不让任何一派独占答案</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>jadeClue</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>virtueMin=60</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>virtue=8;fragments=2;years=-1</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>古灵只留下四字：补天有价。</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>若碎片已足，提前拼合旧约试探轮回边界</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>breakWheel</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>fragmentsMin=4;realmMin=3</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>登潮宫残碑，问东海神域为何沉默</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>jadeClue</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>fragments=1;qi=18;years=-1</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>残碑回答你的不是文字，而是一段被献祭的飞升记忆。</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>救下被当作祭品的神域侍童</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>iceHeart</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>virtueMin=70</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>virtue=22;karma=-10</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>侍童把潮宫暗门告诉你，却求你别把所有神明都当敌人。</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>假意接受神使册封，查九天祭席名单</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>greatCouncil</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>karmaMax=60</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>karma=12;fragments=1</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>你坐上了不该坐的位置，也看清了谁在数人间的命。</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>让心魔代你入梦，偷听祭席背后的交易</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>heartDemon</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>karmaMin=30</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>memory=2;karma=14</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>心魔带回真相，也带回一枚更像你的面具。</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>以修为硬闯九天门缝，先看飞升真假</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>ascend</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>realmMin=5</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>以诸门新约重订绝地天通</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>breakWheel</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>fragmentsMin=4;virtueMin=75</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>因果已重，先入幽都照见本心再谈飞升</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>hell</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>karmaMin=55</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>寿元将尽，把东海神域的坐标交给下一世</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>death</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>yearsMin=1</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>memory=2;fragments=1;years=-99</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>你没有失败，只是把终局推给了更强的自己。</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>以高德行登九天，公开祭席后的旧账</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>ascend</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>realmMin=5;virtueMin=90;karmaMax=45</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>以天命碎片重封铜门，结束献祭式轮回</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>breakWheel</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>fragmentsMin=5;virtueMin=70</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>牺牲本世修为，换诸门凡人全数撤离</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>death</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>virtueMin=100</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>memory=3;fragments=1;qi=-80;years=-99</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>你把胜利留给别人，把答案留给下一世。</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>带着因果强行飞升，赌九天不敢拒你</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>ascend</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>realmMin=6;karmaMin=45</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>若因果压过道心，入幽都重走人间</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>hell</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>karmaMin=65</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>以魍魉、冰心、天机三方证词重审旧约</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>greatCouncil</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>fragmentsMin=3;virtueMin=65</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>virtue=12;karma=-8;memory=1</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>这一次不是你一个人对抗天命，而是大荒一起开口。</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>什么都不争，只把真相刻进轮回记忆</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>death</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>memory=2;fragments=1;years=-99</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>你选择下一世再来，但不是空手而来。</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>若境界已至巅峰，直面东海神域背后的神界边界</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>ascend</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>realmMin=6;fragmentsMin=4</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1061,7 +1903,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
+    <col width="88" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1084,7 +1926,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>你的因果太重，魍魉席后的影子始终盯着你的手。</t>
+          <t>你的因果太重，魍魉席后的影子始终盯着你的手；若再强行登天，幽都会先来要账。</t>
         </is>
       </c>
     </row>
@@ -1096,7 +1938,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>你的名声已足以压住半座议厅，但真正的信任仍要靠下一步换来。</t>
+          <t>你的名声已足以让诸门暂时放下私怨，但真正的信任仍要靠下一步换来。</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1226,6 +2068,752 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ArtPools</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>场景图池。Scene 填网页场景 id，Image 填 assets/*.webp，多个同场景会按随机种子抽一张。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>图片维护</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>新增图片请先压缩为 WebP 放进 assets，再在 ArtPools 增加一行。</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Scene</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Order</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Image</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>birth</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>assets/xiling-ruins.webp</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>初始与西陵旧地</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>birth</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>assets/great-council.webp</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>议厅回忆</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>memoryArchive</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>assets/copper-gate.webp</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>记忆与铜门</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>memoryArchive</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>assets/underworld-ledger.webp</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>轮回档案</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>sect</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>assets/xiling-ruins.webp</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>门派修行</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>iceHeart</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>assets/iceheart-hall.webp</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>冰心堂</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>iceHeart</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>assets/sect-new-pact.webp</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>救人与联盟</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>shadow</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>assets/leize-shadow.webp</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>魍魉影线</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>shadow</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>assets/cold-shadow.webp</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>暗线追查</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>foxRoad</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>assets/fox-road.webp</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>夜路狐影</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>jadeClue</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>assets/east-sea-tide-palace.webp</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>神域线索</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>jadeClue</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>assets/copper-gate.webp</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>铜门裂纹</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>copperGate</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>assets/copper-gate.webp</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>铜门</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>copperGate</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>assets/east-sea-godrealm.webp</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>神域门影</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>northSea</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>assets/beiming-pact.webp</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>北溟旧约</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>northSea</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>assets/beiming-road.webp</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>北溟道路</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>greatCouncil</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>assets/sect-new-pact.webp</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>诸门新约</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>greatCouncil</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>assets/great-council.webp</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>旧议厅</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>tribulation</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>assets/tribulation.webp</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>雷劫破境</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>assets/sect-new-pact.webp</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>阶段推进</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>assets/beiming-pact.webp</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>北溟推进</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>assets/east-sea-tide-palace.webp</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>神域推进</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>heartDemon</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>assets/heart-trial.webp</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>心魔问道</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>heartDemon</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>assets/underworld-ledger.webp</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>因果照见</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>hell</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>assets/underworld-ledger.webp</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>幽都轮回簿</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>hell</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>assets/hell-rebirth.webp</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>幽都重生</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>ascend</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>assets/true-ascend.webp</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>飞升真相</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>ascend</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>assets/east-sea-tide-palace.webp</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>神界边界</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>breakWheel</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>assets/copper-gate.webp</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>重订天通</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>breakWheel</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>assets/sect-new-pact.webp</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>诸门共证</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>trueEnding</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>assets/true-ascend.webp</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>真结局</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>sacrifice</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>assets/copper-gate.webp</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>牺牲封门</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>death</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>assets/xiling-ruins.webp</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>重生回环</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>death</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>assets/underworld-ledger.webp</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>记忆沉淀</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Xuanhui character arc
</commit_message>
<xml_diff>
--- a/story-config.xlsx
+++ b/story-config.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="StatusLines" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ArtPools" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CharacterLore" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -557,18 +558,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="62" customWidth="1" min="9" max="9"/>
+    <col width="66" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -641,20 +642,20 @@
           <t>shadow</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>karma=4;fragments=1</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>魍魉席后一阵沉默。有人承认，铜门裂纹不是第一次出现。</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -673,20 +674,20 @@
           <t>iceHeart</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>virtue=12;years=-1</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>药账里夹着一枚旧印，印文正与铜门边缘吻合。</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -705,7 +706,7 @@
           <t>jadeClue</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="n"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>fragments=1;qi=10</t>
@@ -716,13 +717,13 @@
           <t>是</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
           <t>机关鸟飞回时，爪上多了一粒东海盐晶。</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -751,14 +752,14 @@
           <t>virtue=6;karma=6;fragments=1</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
           <t>封锁不是仁慈，却让三个说谎的人同时露怯。</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -777,7 +778,7 @@
           <t>tribulation</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>qi=18;years=-1</t>
@@ -788,13 +789,13 @@
           <t>是</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="n"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
           <t>星图尽头不是九天，而是一片被抹去名字的海。</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -813,20 +814,20 @@
           <t>copperGate</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
           <t>qi=22;karma=6;years=-1</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr"/>
-      <c r="H7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="inlineStr">
         <is>
           <t>沉船铁锈里藏着神域火纹，像是专为破门而铸。</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -845,81 +846,85 @@
           <t>foxRoad</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>memory=1;karma=3</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="inlineStr">
         <is>
           <t>影步尽头留着半句誓词：救人者也会成为钥匙。</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>公开天书残页，迫诸门当场站队</t>
+          <t>追上自称玄晖的旅人，问他为何独往北溟</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>greatCouncil</t>
+          <t>northSea</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>virtue=8;karma=3</t>
+          <t>xuanhuiBond=1;sunCinders=1;fragments=1;years=-1</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
       <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>诸门终于不再谈风骨，只开始谈各自欠下的债。</t>
+          <t>玄晖不答，只说北溟有一个人欠他答案。水镜里一瞬映出十轮残日。</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B10" s="2" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>夜入北溟，追玄晶留下的幽都旧约</t>
+          <t>替玄晖挡下天机营盘问，只记下他的金色瞳纹</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>northSea</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
+          <t>foxRoad</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>karmaMax=35</t>
+        </is>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>fragments=1;years=-1</t>
+          <t>xuanhuiBond=2;virtue=4;sunCinders=1</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
       <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>北溟风雪里，你听见幽都并不承认自己是地狱。</t>
+          <t>他第一次认真看你，像在确认你是否把失势神子也当作活人。</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
@@ -929,94 +934,86 @@
         <v>1</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>独自贴近铜门，听清门内喊出的名字</t>
+          <t>公开天书残页，迫诸门当场站队</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>copperGate</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr"/>
+          <t>greatCouncil</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>qi=16;karma=8</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr"/>
+          <t>virtue=8;karma=3</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>铜门没有打开，只把你的倒影换成了上一世的样子。</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr"/>
+          <t>诸门终于不再谈风骨，只开始谈各自欠下的债。</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
         <v>1</v>
       </c>
       <c r="B12" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>请冰心堂先验疫民魂灯，查谁动过生死簿</t>
+          <t>夜入北溟，追玄晶留下的幽都旧约</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>iceHeart</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>virtueMin=55</t>
-        </is>
-      </c>
+          <t>northSea</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>virtue=14;fragments=1;years=-1</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr"/>
-      <c r="H12" s="2" t="inlineStr"/>
+          <t>fragments=1;years=-1</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>魂灯没有灭，说明有人把活人提前写进了死册。</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr"/>
+          <t>北溟风雪里，你听见幽都并不承认自己是地狱。</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
         <v>1</v>
       </c>
       <c r="B13" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>与弈剑旧友论剑三夜，换他带你进旧阵眼</t>
+          <t>独自贴近铜门，听清门内喊出的名字</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>tribulation</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
+          <t>copperGate</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>qi=24;years=-2</t>
+          <t>qi=16;karma=8</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1024,222 +1021,222 @@
           <t>是</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>剑意洗去浮躁，也削开阵眼外层的伪装。</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr"/>
+          <t>铜门没有打开，只把你的倒影换成了上一世的样子。</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
         <v>1</v>
       </c>
       <c r="B14" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>让魍魉暗网散出假消息，引蛇出洞</t>
+          <t>请冰心堂先验疫民魂灯，查谁动过生死簿</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>shadow</t>
+          <t>iceHeart</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>karmaMax=45</t>
+          <t>virtueMin=55</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>karma=9;fragments=1</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr"/>
-      <c r="H14" s="2" t="inlineStr"/>
+          <t>virtue=14;fragments=1;years=-1</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>这不是作恶，是用影子照出更深的影子。</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr"/>
+          <t>魂灯没有灭，说明有人把活人提前写进了死册。</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
         <v>1</v>
       </c>
       <c r="B15" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>护送一队凡人离开裂隙，暂缓追查</t>
+          <t>与弈剑旧友论剑三夜，换他带你进旧阵眼</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>death</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>yearsMin=1;virtueMin=80</t>
-        </is>
-      </c>
+          <t>tribulation</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>virtue=18;memory=1;years=-1</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr"/>
-      <c r="H15" s="2" t="inlineStr"/>
+          <t>qi=24;years=-2</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>他们不知道真相，却会在下一世替你记得一个名字。</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr"/>
+          <t>剑意洗去浮躁，也削开阵眼外层的伪装。</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B16" s="2" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>把北溟旧约带回议厅，要求诸门共证</t>
+          <t>让魍魉暗网散出假消息，引蛇出洞</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>greatCouncil</t>
+          <t>shadow</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>fragmentsMin=2</t>
+          <t>karmaMax=45</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>virtue=10;karma=5</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr"/>
-      <c r="H16" s="2" t="inlineStr"/>
+          <t>karma=9;fragments=1</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>旧约一出，最先拔剑的不是魔修，而是仙盟使者。</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr"/>
+          <t>这不是作恶，是用影子照出更深的影子。</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B17" s="2" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>潜入幽都边市，查轮回簿被谁改写</t>
+          <t>护送一队凡人离开裂隙，暂缓追查</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>hell</t>
+          <t>death</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>karmaMin=45</t>
+          <t>yearsMin=1;virtueMin=80</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>memory=2;karma=-8</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr"/>
-      <c r="H17" s="2" t="inlineStr"/>
+          <t>virtue=18;memory=1;years=-1</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>幽都没有审你，只让你看见自己每次逃避的代价。</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="inlineStr"/>
+          <t>他们不知道真相，却会在下一世替你记得一个名字。</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B18" s="2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>闭关炼化盐晶，冲击更高境界</t>
+          <t>查玄晖留在药账里的乌羽灰</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>tribulation</t>
+          <t>iceHeart</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>qi=38;years=-2</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
+          <t>xuanhuiBond=1;sunCinders=2;virtue=6</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>盐晶化作潮声，丹田里第一次出现神域门影。</t>
+          <t>乌羽灰遇药灯不燃，反而照出灵巫宫旧歌里的东君日轮。</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>救北溟雪灾里的敌派弟子，不问立场</t>
+          <t>把玄晖的旧名交给诸门，换取东皇太一档案</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>iceHeart</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
+          <t>greatCouncil</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>karmaMax=50</t>
+        </is>
+      </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>virtue=20;karma=-6;years=-1</t>
+          <t>sunCinders=2;karma=8;xuanhuiBond=-1</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
       <c r="H19" s="2" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>对方醒来后只说一句：原来你不是为了赢。</t>
+          <t>诸门只听见东皇太一四字，没人问玄晖为何宁愿用人间化名。</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr"/>
@@ -1249,335 +1246,351 @@
         <v>2</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>借荒火战阵强行撬开铜门外环</t>
+          <t>把北溟旧约带回议厅，要求诸门共证</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>copperGate</t>
+          <t>greatCouncil</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>realmMin=2</t>
+          <t>fragmentsMin=2</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>qi=30;karma=12;fragments=1;years=-2</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr"/>
-      <c r="H20" s="2" t="inlineStr"/>
+          <t>virtue=10;karma=5</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>铜门震动，九天祭席上有一个无名位被点亮。</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr"/>
+          <t>旧约一出，最先拔剑的不是魔修，而是仙盟使者。</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
         <v>2</v>
       </c>
       <c r="B21" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>用魍魉影契换取神域使者真名</t>
+          <t>潜入幽都边市，查轮回簿被谁改写</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>heartDemon</t>
+          <t>hell</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>karmaMin=20</t>
+          <t>karmaMin=45</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>fragments=1;karma=10;memory=1</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="inlineStr"/>
-      <c r="H21" s="2" t="inlineStr"/>
+          <t>memory=2;karma=-8</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>你得到了真名，也听见心魔学会了那人的声音。</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr"/>
+          <t>幽都没有审你，只让你看见自己每次逃避的代价。</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
         <v>2</v>
       </c>
       <c r="B22" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>请太虚观召灵问古，不让任何一派独占答案</t>
+          <t>闭关炼化盐晶，冲击更高境界</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>jadeClue</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>virtueMin=60</t>
-        </is>
-      </c>
+          <t>tribulation</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>virtue=8;fragments=2;years=-1</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr"/>
-      <c r="H22" s="2" t="inlineStr"/>
+          <t>qi=38;years=-2</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n"/>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>古灵只留下四字：补天有价。</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr"/>
+          <t>盐晶化作潮声，丹田里第一次出现神域门影。</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
         <v>2</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>若碎片已足，提前拼合旧约试探轮回边界</t>
+          <t>救北溟雪灾里的敌派弟子，不问立场</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>breakWheel</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>fragmentsMin=4;realmMin=3</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="inlineStr"/>
-      <c r="H23" s="2" t="inlineStr"/>
-      <c r="I23" s="2" t="inlineStr"/>
-      <c r="J23" s="2" t="inlineStr"/>
+          <t>iceHeart</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>virtue=20;karma=-6;years=-1</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>对方醒来后只说一句：原来你不是为了赢。</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>登潮宫残碑，问东海神域为何沉默</t>
+          <t>借荒火战阵强行撬开铜门外环</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>jadeClue</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr"/>
+          <t>copperGate</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>realmMin=2</t>
+        </is>
+      </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>fragments=1;qi=18;years=-1</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr"/>
+          <t>qi=30;karma=12;fragments=1;years=-2</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n"/>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>残碑回答你的不是文字，而是一段被献祭的飞升记忆。</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr"/>
+          <t>铜门震动，九天祭席上有一个无名位被点亮。</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>救下被当作祭品的神域侍童</t>
+          <t>用魍魉影契换取神域使者真名</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>iceHeart</t>
+          <t>heartDemon</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>virtueMin=70</t>
+          <t>karmaMin=20</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>virtue=22;karma=-10</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr"/>
-      <c r="H25" s="2" t="inlineStr"/>
+          <t>fragments=1;karma=10;memory=1</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n"/>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>侍童把潮宫暗门告诉你，却求你别把所有神明都当敌人。</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr"/>
+          <t>你得到了真名，也听见心魔学会了那人的声音。</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B26" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>假意接受神使册封，查九天祭席名单</t>
+          <t>请太虚观召灵问古，不让任何一派独占答案</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>greatCouncil</t>
+          <t>jadeClue</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>karmaMax=60</t>
+          <t>virtueMin=60</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>karma=12;fragments=1</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
+          <t>virtue=8;fragments=2;years=-1</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>你坐上了不该坐的位置，也看清了谁在数人间的命。</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr"/>
+          <t>古灵只留下四字：补天有价。</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>让心魔代你入梦，偷听祭席背后的交易</t>
+          <t>若碎片已足，提前拼合旧约试探轮回边界</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>heartDemon</t>
+          <t>breakWheel</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>karmaMin=30</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>memory=2;karma=14</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr"/>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>心魔带回真相，也带回一枚更像你的面具。</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr"/>
+          <t>fragmentsMin=4;realmMin=3</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="2" t="n"/>
+      <c r="I27" s="2" t="n"/>
+      <c r="J27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B28" s="2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>以修为硬闯九天门缝，先看飞升真假</t>
+          <t>在北溟雪夜听玄晖讲射日之后</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>ascend</t>
+          <t>northSea</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>realmMin=5</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr"/>
+          <t>xuanhuiBondMin=2</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>xuanhuiBond=2;sunCinders=2;memory=1;years=-1</t>
+        </is>
+      </c>
       <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr"/>
-      <c r="I28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>他说十日坠落时，他才知道贵为神明也会被命运写定。</t>
+        </is>
+      </c>
       <c r="J28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B29" s="2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>以诸门新约重订绝地天通</t>
+          <t>帮玄晖摆脱化生魔禁制，换他借金乌火炼契</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>breakWheel</t>
+          <t>tribulation</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>fragmentsMin=4;virtueMin=75</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr"/>
-      <c r="G29" s="2" t="inlineStr"/>
+          <t>sunCindersMin=3</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>qi=32;karma=6;sunCinders=1;xuanhuiBond=1</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
       <c r="H29" s="2" t="inlineStr"/>
-      <c r="I29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>金乌火没有焚尽幽都，只烧掉了旧契上最不肯见人的一角。</t>
+        </is>
+      </c>
       <c r="J29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
@@ -1585,195 +1598,211 @@
         <v>3</v>
       </c>
       <c r="B30" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>因果已重，先入幽都照见本心再谈飞升</t>
+          <t>登潮宫残碑，问东海神域为何沉默</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>hell</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>karmaMin=55</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr"/>
-      <c r="G30" s="2" t="inlineStr"/>
-      <c r="H30" s="2" t="inlineStr"/>
-      <c r="I30" s="2" t="inlineStr"/>
-      <c r="J30" s="2" t="inlineStr"/>
+          <t>jadeClue</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>fragments=1;qi=18;years=-1</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>残碑回答你的不是文字，而是一段被献祭的飞升记忆。</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
         <v>3</v>
       </c>
       <c r="B31" s="2" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>寿元将尽，把东海神域的坐标交给下一世</t>
+          <t>救下被当作祭品的神域侍童</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>death</t>
+          <t>iceHeart</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>yearsMin=1</t>
+          <t>virtueMin=70</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>memory=2;fragments=1;years=-99</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr"/>
-      <c r="H31" s="2" t="inlineStr"/>
+          <t>virtue=22;karma=-10</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n"/>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>你没有失败，只是把终局推给了更强的自己。</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr"/>
+          <t>侍童把潮宫暗门告诉你，却求你别把所有神明都当敌人。</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B32" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>以高德行登九天，公开祭席后的旧账</t>
+          <t>假意接受神使册封，查九天祭席名单</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>ascend</t>
+          <t>greatCouncil</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>realmMin=5;virtueMin=90;karmaMax=45</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="inlineStr"/>
-      <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr"/>
+          <t>karmaMax=60</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>karma=12;fragments=1</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>你坐上了不该坐的位置，也看清了谁在数人间的命。</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B33" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B33" s="2" t="n">
-        <v>2</v>
-      </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>以天命碎片重封铜门，结束献祭式轮回</t>
+          <t>让心魔代你入梦，偷听祭席背后的交易</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>breakWheel</t>
+          <t>heartDemon</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>fragmentsMin=5;virtueMin=70</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr"/>
-      <c r="G33" s="2" t="inlineStr"/>
-      <c r="H33" s="2" t="inlineStr"/>
-      <c r="I33" s="2" t="inlineStr"/>
-      <c r="J33" s="2" t="inlineStr"/>
+          <t>karmaMin=30</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>memory=2;karma=14</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>心魔带回真相，也带回一枚更像你的面具。</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B34" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>牺牲本世修为，换诸门凡人全数撤离</t>
+          <t>以修为硬闯九天门缝，先看飞升真假</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>death</t>
+          <t>ascend</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>virtueMin=100</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>memory=3;fragments=1;qi=-80;years=-99</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr"/>
-      <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>你把胜利留给别人，把答案留给下一世。</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr"/>
+          <t>realmMin=5</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+      <c r="I34" s="2" t="n"/>
+      <c r="J34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B35" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>带着因果强行飞升，赌九天不敢拒你</t>
+          <t>以诸门新约重订绝地天通</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>ascend</t>
+          <t>breakWheel</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>realmMin=6;karmaMin=45</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" s="2" t="inlineStr"/>
-      <c r="H35" s="2" t="inlineStr"/>
-      <c r="I35" s="2" t="inlineStr"/>
-      <c r="J35" s="2" t="inlineStr"/>
+          <t>fragmentsMin=4;virtueMin=75</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
+      <c r="I35" s="2" t="n"/>
+      <c r="J35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B36" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>若因果压过道心，入幽都重走人间</t>
+          <t>因果已重，先入幽都照见本心再谈飞升</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1783,110 +1812,442 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>karmaMin=65</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="2" t="inlineStr"/>
-      <c r="H36" s="2" t="inlineStr"/>
-      <c r="I36" s="2" t="inlineStr"/>
-      <c r="J36" s="2" t="inlineStr"/>
+          <t>karmaMin=55</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="n"/>
+      <c r="G36" s="2" t="n"/>
+      <c r="H36" s="2" t="n"/>
+      <c r="I36" s="2" t="n"/>
+      <c r="J36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B37" s="2" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>以魍魉、冰心、天机三方证词重审旧约</t>
+          <t>寿元将尽，把东海神域的坐标交给下一世</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>greatCouncil</t>
+          <t>death</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>fragmentsMin=3;virtueMin=65</t>
+          <t>yearsMin=1</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>virtue=12;karma=-8;memory=1</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr"/>
-      <c r="H37" s="2" t="inlineStr"/>
+          <t>memory=2;fragments=1;years=-99</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="n"/>
+      <c r="H37" s="2" t="n"/>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>这一次不是你一个人对抗天命，而是大荒一起开口。</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr"/>
+          <t>你没有失败，只是把终局推给了更强的自己。</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B38" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>什么都不争，只把真相刻进轮回记忆</t>
+          <t>陪玄晖去见幽都王颛顼，哪怕再次被拒</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>death</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr"/>
+          <t>hell</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>xuanhuiBondMin=4</t>
+        </is>
+      </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>memory=2;fragments=1;years=-99</t>
+          <t>xuanhuiBond=2;sunCinders=1;memory=1;karma=-4</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="2" t="inlineStr"/>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>你选择下一世再来，但不是空手而来。</t>
+          <t>颛顼没有开门。玄晖站在门外很久，仍没有低头。</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B39" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>若境界已至巅峰，直面东海神域背后的神界边界</t>
+          <t>释放金乌烬，让十日残光照穿神域祭席</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>ascend</t>
+          <t>heartDemon</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>realmMin=6;fragmentsMin=4</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr"/>
+          <t>sunCindersMin=5</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>fragments=1;sunCinders=2;karma=10</t>
+        </is>
+      </c>
       <c r="G39" s="2" t="inlineStr"/>
       <c r="H39" s="2" t="inlineStr"/>
-      <c r="I39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>十道残光照出九天祭席后的空名，你也听见心魔学会了神的语气。</t>
+        </is>
+      </c>
       <c r="J39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>以高德行登九天，公开祭席后的旧账</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>ascend</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>realmMin=5;virtueMin=90;karmaMax=45</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="n"/>
+      <c r="G40" s="2" t="n"/>
+      <c r="H40" s="2" t="n"/>
+      <c r="I40" s="2" t="n"/>
+      <c r="J40" s="2" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>以天命碎片重封铜门，结束献祭式轮回</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>breakWheel</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>fragmentsMin=5;virtueMin=70</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="n"/>
+      <c r="G41" s="2" t="n"/>
+      <c r="H41" s="2" t="n"/>
+      <c r="I41" s="2" t="n"/>
+      <c r="J41" s="2" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B42" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>牺牲本世修为，换诸门凡人全数撤离</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>death</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>virtueMin=100</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>memory=3;fragments=1;qi=-80;years=-99</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="n"/>
+      <c r="H42" s="2" t="n"/>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>你把胜利留给别人，把答案留给下一世。</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>带着因果强行飞升，赌九天不敢拒你</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>ascend</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>realmMin=6;karmaMin=45</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="n"/>
+      <c r="H43" s="2" t="n"/>
+      <c r="I43" s="2" t="n"/>
+      <c r="J43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B44" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>若因果压过道心，入幽都重走人间</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>hell</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>karmaMin=65</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="n"/>
+      <c r="G44" s="2" t="n"/>
+      <c r="H44" s="2" t="n"/>
+      <c r="I44" s="2" t="n"/>
+      <c r="J44" s="2" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B45" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>以魍魉、冰心、天机三方证词重审旧约</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>greatCouncil</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>fragmentsMin=3;virtueMin=65</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>virtue=12;karma=-8;memory=1</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="n"/>
+      <c r="H45" s="2" t="n"/>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>这一次不是你一个人对抗天命，而是大荒一起开口。</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B46" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>什么都不争，只把真相刻进轮回记忆</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>death</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="n"/>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>memory=2;fragments=1;years=-99</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="n"/>
+      <c r="H46" s="2" t="n"/>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>你选择下一世再来，但不是空手而来。</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B47" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>若境界已至巅峰，直面东海神域背后的神界边界</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>ascend</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>realmMin=6;fragmentsMin=4</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="n"/>
+      <c r="G47" s="2" t="n"/>
+      <c r="H47" s="2" t="n"/>
+      <c r="I47" s="2" t="n"/>
+      <c r="J47" s="2" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B48" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>以玄晖之名重写东皇旧契：神子也有选择命运的权利</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>breakWheel</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>xuanhuiBondMin=6;sunCindersMin=6;virtueMin=70</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>virtue=18;fragments=1;memory=2</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>玄晖没有登回神座。他把最后一缕金乌火交给人间诸门共守。</t>
+        </is>
+      </c>
+      <c r="J48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B49" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>强迫玄晖归位东皇，以十日之火焚开天门</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>ascend</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>sunCindersMin=6;karmaMin=35</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>qi=60;karma=24;xuanhuiBond=-3</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr"/>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>十日同升，天门大开。可你分不清那是飞升，还是又一次把他献上祭席。</t>
+        </is>
+      </c>
+      <c r="J49" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1965,7 +2326,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2089,6 +2450,18 @@
       <c r="B10" t="inlineStr">
         <is>
           <t>新增图片请先压缩为 WebP 放进 assets，再在 ArtPools 增加一行。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>人物线</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CharacterLore 记录人物设定；Choices 可使用 xuanhuiBond / sunCinders 等数值做 Effects 和 Requires。</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2814,6 +3187,238 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>northSea</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>assets/xuanhui-beiming.webp</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>玄晖北溟寻父</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>hell</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>3</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>assets/xuanhui-beiming.webp</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>颛顼拒见与幽都门</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>heartDemon</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>3</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>assets/xuanhui-beiming.webp</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>十日旧劫心魔</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Character</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>玄晖</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>文档依据</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>大荒人物志：东皇太一失去力量后，以人类身份行动，取化名玄晖；玄为天，晖为日，玄晖即太阳别称。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>东皇太一</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>身世</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>大荒人物志：东皇太一是帝江之子、十日之首；帝俊对外宣称太阳十子为自己和羲和之子，并遮蔽真实身世。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>十日旧劫</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>射日之后</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>大荒人物志：太阳十子得知帝俊与帝江真相后化为金乌炙烤大地，最终被射落；太一在坠落时意识到自己的命运早被安排。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>北溟寻父</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>人物动机</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>大荒人物志：太一想找到生父帝江，也就是如今的幽都王颛顼；但颛顼拒绝回答，也拒绝提供面见机会。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>玄晖</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>人物线定位</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>本游戏把玄晖线写成人性与神格的冲突：尊重玄晖作为人的选择会提升玄晖缘，逼迫他归位东皇会提升力量但增加因果。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>金乌十日</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>母题线</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>天下，我们的大荒：帝俊、帝江、东皇太一皆可视为东夷太阳图腾脉络；游戏以金乌烬表现十日旧劫残留。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>数值</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>xuanhuiBond</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>玄晖缘。代表玩家理解、保护、尊重玄晖作为人的程度。高值开放新约/真结局辅助线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>数值</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>sunCinders</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>金乌烬。代表玩家触及东皇太一与十日旧劫真相的深度。高值开放强力但高风险选项。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Move story revelations into life verdicts
</commit_message>
<xml_diff>
--- a/story-config.xlsx
+++ b/story-config.xlsx
@@ -482,9 +482,9 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>你睁眼时，手心攥着一小片温热的铜锈。
-窗外不是同一个清晨。有人在西陵废墙下哭，有人在雷泽雾里点灯，也有人把一盏药炉搬到你床前。
+窗外不是同一个清晨。有人在废墙下哭，有人在雾里点灯，也有人把药炉搬到你床前。
 {{status}}
-这一世先从哪里开始，会决定谁最早看见你。</t>
+先活下去。至于这一世会遇见谁，还要等你走出去。</t>
         </is>
       </c>
     </row>
@@ -500,9 +500,9 @@
       <c r="C3" t="inlineStr">
         <is>
           <t>十二岁到十六岁之间，你终于被大荒某一扇门接住。
-门规、药账、剑匣、星图、邪影、暗网、机关鸟、试锋石，都把你的名字写进不同的册子。
+有人递给你盾，有人递给你药杵，有人只把剑匣推到桌边，让你自己打开。
 {{status}}
-入门不是归宿，只是第一笔因果。</t>
+门里没有答案，只有第一条规矩。</t>
         </is>
       </c>
     </row>
@@ -517,10 +517,10 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>第一次下山，你发现每个传闻背后都有一个活人。
-书生袖中藏着九尾，药童掌心结着寒霜，魔女桌上放着旧药瓶，北溟旅人把手伸进火里。
+          <t>第一次下山，雨从屋檐滴到刀鞘上。
+你在城门、药庐、山道和雪线边遇见不同的人。他们都像路过，却都没有真的走开。
 {{status}}
-你可以利用他们，也可以先听他们把话说完。</t>
+这一回，先听谁把话说完？</t>
         </is>
       </c>
     </row>
@@ -536,9 +536,9 @@
       <c r="C5" t="inlineStr">
         <is>
           <t>弈剑旧阁的雨下了三日。
-剑匣自己开了一线，里面不是剑光，而是一卷被虫蛀穿的《玄华名剑录》。每一页都贴着一段人命。
+剑匣自己开了一线，里面不是剑光，而是一卷被虫蛀穿的旧录。纸页潮湿，边角还沾着干血。
 {{status}}
-从黄泉到碧落，有些剑只是在路过人间时出了鞘。</t>
+你伸手时，匣中传来第二个人的呼吸。</t>
         </is>
       </c>
     </row>
@@ -554,9 +554,9 @@
       <c r="C6" t="inlineStr">
         <is>
           <t>北溟雪线尽头，潮声从冰下传来。
-玄晖的脚印里有金乌灰，东海残碑上有少昊旧名，幽都门前却只挂着一盏不肯灭的灯。
+雪地里有一串脚印，脚印旁落着不融的金灰。远处的门关着，门前有灯。
 {{status}}
-这一幕开始，神话不再是书上的旧事。</t>
+你还不知道门后是谁，只知道有人已经等得太久。</t>
         </is>
       </c>
     </row>
@@ -566,15 +566,15 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>三界旧契</t>
+          <t>水镜前的证词</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>你把证据摆在水镜前：药账、白羽、六翼令、青阳痕、上邪残锋、金乌烬。
-镜中先映出黄泉，再映出碧落，最后映出你这一世救过又没救成的人。
+          <t>你把这一世带回来的东西摆在水镜前。
+药账、白羽、残锋、盐晶、六翼令，每一样都很轻，放在桌上却压得众人沉默。
 {{status}}
-三界都在问你，要不要继续把人间当路。</t>
+现在轮到他们解释了。</t>
         </is>
       </c>
     </row>
@@ -590,8 +590,8 @@
       <c r="C8" t="inlineStr">
         <is>
           <t>铜门前没有风。
-诸门站在你身后，幽都在门下沉默，九天祭席上亮着一排名字，其中有你的，也有你这一世认识过的所有人。
-道德越稳，越有人愿意替你作证；因果越重，幽都越早照见你。现在该结账了。</t>
+你听见身后有人拔剑，有人点灯，有人低声念你的名字。门上的铜锈一点点发热。
+这一世走到这里，已经没有旁观的位置。</t>
         </is>
       </c>
     </row>
@@ -690,13 +690,11 @@
           <t>greatCouncil</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>virtue=8;memory=1;years=-1</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>天机营</t>
@@ -707,7 +705,6 @@
           <t>孩子的手印沾在天机盾背面。你还不知道他的名字，却已经知道这一世不能只顾修行。</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -726,13 +723,11 @@
           <t>iceHeart</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>virtue=6;iceLedger=1;years=-1</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>冰心堂</t>
@@ -743,7 +738,6 @@
           <t>清时把药账翻到最后一页。一个三年前死在西陵的人，被写成明日午时入炉。</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -762,13 +756,11 @@
           <t>shadow</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>karma=3;shadowTrust=1;memory=1</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>魍魉</t>
@@ -779,7 +771,6 @@
           <t>夜哭没有回头，只把一枚六翼令丢进水里。令牌没有沉，反而映出你的脸。</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -798,7 +789,6 @@
           <t>jadeClue</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>fragments=1;qi=12;moFeiyunProof=1;years=-1</t>
@@ -819,7 +809,6 @@
           <t>星图尽头不是九天，而是一片被抹去名字的海。莫非云在页角夹了一根白羽。</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -838,7 +827,6 @@
           <t>tribulation</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>swordHeart=1;qingyangTrace=1;qi=10</t>
@@ -859,7 +847,6 @@
           <t>雨水从剑匣缝里往上流。弈剑客说：从黄泉到碧落，我只是路过人间。</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -878,7 +865,6 @@
           <t>jadeClue</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>inkContract=1;fragments=1;qi=8</t>
@@ -899,7 +885,6 @@
           <t>遗墨把机关鸟递给你，鸟腹里滚出一粒盐晶，晶面刻着你的上一世生辰。</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -918,13 +903,11 @@
           <t>copperGate</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>fireOath=1;qi=18;karma=5;years=-1</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>荒火教</t>
@@ -935,7 +918,6 @@
           <t>彤把长刀插进地里，问你火是用来开路，还是用来烧尽挡路的人。</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -954,13 +936,11 @@
           <t>foxRoad</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>foxBond=1;virtue=7;memory=1</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>青丘客</t>
@@ -971,7 +951,6 @@
           <t>书生皱着眉，像是不明白自己为什么停下。火光里，九道白影一闪即逝。</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1000,7 +979,6 @@
           <t>xuanhuiBond=2;sunCinders=1;virtue=4;years=-1</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>北溟客</t>
@@ -1011,7 +989,6 @@
           <t>追魂符落在雪上不燃。玄晖看了你很久，说：你认错人了，我只是路过。</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1040,7 +1017,6 @@
           <t>memory=2;karma=-5;years=-1</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>幽都照影</t>
@@ -1051,7 +1027,6 @@
           <t>判官没有锁链，只把灯推到你面前。灯里照出的是你上一世没救走的人。</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1070,13 +1045,11 @@
           <t>greatCouncil</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>virtue=10;fragments=1;years=-1</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>天机营</t>
@@ -1087,7 +1060,6 @@
           <t>营官说军册只记战功。你把盾背翻给他看，满厅忽然没人说话。</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1106,13 +1078,11 @@
           <t>iceHeart</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>iceLedger=2;virtue=8;karma=3;fragments=1</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>冰心堂</t>
@@ -1123,7 +1093,6 @@
           <t>清时的寒霜爬上账页。被写进死册的活人，正在门外排队取药。</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1142,7 +1111,6 @@
           <t>tribulation</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>swordHeart=2;qingyangTrace=1;qi=22;years=-1</t>
@@ -1163,7 +1131,6 @@
           <t>第三剑没有落在你身上，而是斩开雨幕。阵眼下露出四字：青阳降居。</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1182,13 +1149,11 @@
           <t>jadeClue</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>moFeiyunProof=2;virtue=6;fragments=1</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>云麓仙居</t>
@@ -1199,7 +1164,6 @@
           <t>莫非云把白羽压在残页上。羽尖指向的不是太虚，是云麓一枚旧私印。</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1218,13 +1182,11 @@
           <t>heartDemon</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>shadowTrust=1;memory=1;karma=-2</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>太虚观</t>
@@ -1235,7 +1197,6 @@
           <t>镜中邪影没有扑来，只学你的声音问：若被污名的是你，你还信门规吗？</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1254,13 +1215,11 @@
           <t>shadow</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>shadowTrust=2;karma=4;fragments=1</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>魍魉</t>
@@ -1271,7 +1230,6 @@
           <t>长老们在岸上争血统。你潜进水底，只看见令牌旁有一道替人挡刀的旧痕。</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1290,7 +1248,6 @@
           <t>jadeClue</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>inkContract=2;fragments=1;qi=10;years=-1</t>
@@ -1311,7 +1268,6 @@
           <t>机关鸟起飞前回头看了遗墨一眼，像一个不善告别的人。</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1330,13 +1286,11 @@
           <t>copperGate</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>fireOath=2;virtue=5;qi=20;karma=2</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>荒火教</t>
@@ -1347,7 +1301,6 @@
           <t>石裂三寸，地底传来笑声。彤握紧刀柄，说这把火还不到交给疯子的时候。</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1366,13 +1319,11 @@
           <t>foxRoad</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>foxBond=2;virtue=8;memory=1</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>天机营</t>
@@ -1383,7 +1334,6 @@
           <t>他把尾影藏进袖里，偏偏在妖魔冲阵时忘了藏。九道狐火照亮盾墙。</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1412,7 +1362,6 @@
           <t>swordHeart=1;fragments=1;karma=2</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>弈剑听雨阁</t>
@@ -1423,7 +1372,6 @@
           <t>残页割破手指。血落在上邪二字旁，纸页里传来黄泉水声。</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1452,14 +1400,11 @@
           <t>iceLedger=1;virtue=14;karma=-4;years=-1</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>清时没有道谢。他只是把毒针收回袖中，替敌将把断气接了回来。</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1488,14 +1433,11 @@
           <t>moFeiyunProof=1;shadowTrust=1;virtue=8;karma=-3</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>冷喻没有哭。她把白羽压在旧药瓶下，瓶底云麓私印终于露出来。</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1524,14 +1466,11 @@
           <t>foxBond=2;virtue=10;years=-1</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>天快亮时，他问你：若我今日怕死，还算不算懂了人间感情？</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1550,20 +1489,16 @@
           <t>northSea</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>xuanhuiBond=2;sunCinders=1;virtue=5</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>火没有烧他，却把你的掌心烫出一圈残日。他低声说：神子也会冷。</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1592,14 +1527,11 @@
           <t>shadowTrust=2;virtue=6;karma=2;fragments=1</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>夜哭看着那两道墨痕，第一次说：影子不是谁都杀。</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1628,14 +1560,11 @@
           <t>inkContract=2;virtue=12;fragments=1;years=-1</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
           <t>机关鸟载不动所有人。遗墨拆下自己的剑炉，把第二只鸟拼到天亮。</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1669,13 +1598,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>彤背对殿门站了很久。她说荒火可以输，但不能把人间交给一场疯火。</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1704,14 +1631,11 @@
           <t>swordHeart=2;qingyangTrace=1;memory=1</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>他擦剑的手停了一下：因为停得太久，就会以为黄泉和碧落都比人间重要。</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1740,14 +1664,11 @@
           <t>moFeiyunProof=1;virtue=10;karma=4;fragments=1</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
           <t>星图亮起时，云麓长老先拔剑斩镜。你看见他怕的不是魔女，是证词。</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1776,14 +1697,11 @@
           <t>xuanhuiBond=2;sunCinders=2;memory=1;years=-1</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
           <t>他说十日坠落时，他才知道贵为神明也会被写进别人的命数。</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1812,14 +1730,11 @@
           <t>memory=2;virtue=6;years=-99</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
           <t>这一世你没有走到铜门前。但下一世，你会更早认出他们。</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1853,13 +1768,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
           <t>创派之剑没有剑鸣，只有广成子旧印。黄帝帝师四字，被雨水泡得发白。</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1893,13 +1806,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
           <t>残纹尽头接着东海潮声。少昊的名字在水里一闪，像被谁故意抹去。</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1928,14 +1839,11 @@
           <t>virtue=12;fragments=1;iceLedger=1</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
           <t>剑没有出鞘，只横在两本册子之间。先低头的是拿军令的人。</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1954,20 +1862,16 @@
           <t>heartDemon</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>fragments=1;karma=8;memory=1</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
-      <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
           <t>黑玄剑影里没有狂笑，只有一张排满名字的棋盘。最边上，是你的字迹。</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1986,20 +1890,16 @@
           <t>hell</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>memory=1;karma=5;fragments=1</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
           <t>残锋贴近耳边时，黄泉水忽然涨潮。有人抱剑发誓，终有一日踏破九黎。</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2028,14 +1928,11 @@
           <t>virtue=14;shadowTrust=1;fragments=1</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
           <t>桃木剑轻得像玩具，却斩断了药瓶上的假封条。满厅没有一个人敢笑。</t>
         </is>
       </c>
-      <c r="J38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2054,20 +1951,16 @@
           <t>iceHeart</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>moFeiyunProof=1;iceLedger=1;karma=3;fragments=1</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
           <t>情毒二字下压着两枚印：一枚云麓，一枚太虚。莫非云的白羽夹在中间。</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2096,14 +1989,11 @@
           <t>swordHeart=2;fragments=1;karma=4</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>龙渊映出的不是神座，是一排空名。每个空名旁都放着一盏人间魂灯。</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2137,13 +2027,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
           <t>火里浮出的神纹歪了一笔。弈剑客笑了：仿得这么急，看来九天也会怕。</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2172,14 +2060,11 @@
           <t>memory=3;swordHeart=1;fragments=1;years=-99</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>你合上剑录时，听见剑匣里那第二道呼吸终于平稳下来。</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2208,14 +2093,11 @@
           <t>qingyangTrace=2;fragments=2;years=-1</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
           <t>残碑没有回答，只把黄帝飞升那日的潮声还给你。</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2244,14 +2126,11 @@
           <t>xuanhuiBond=2;sunCinders=1;memory=1;karma=-4</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
           <t>门没有开。玄晖站到雪停，仍没有低头。你第一次觉得沉默也是一种拒绝。</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2280,14 +2159,11 @@
           <t>memory=2;karma=-8;fragments=1</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
           <t>判官收下残锋，却没有笑。他说黄泉不缺恨，缺的是肯认账的人。</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2316,14 +2192,11 @@
           <t>sunCinders=2;fragments=1;karma=8</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr"/>
-      <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
           <t>潮宫地面亮起十个空圈。玄晖只看第一个，像看一张早被烧掉的家谱。</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2352,14 +2225,11 @@
           <t>foxBond=1;virtue=16;karma=-4;years=-1</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
           <t>狐火不烫，落在孩子肩上像一小片春天。九尾却冻得脸色发白。</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2388,14 +2258,11 @@
           <t>shadowTrust=1;memory=2;karma=6;fragments=1</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
           <t>夜哭回来时袖口结霜。他只带回一句话：你的死期，不止被改过一次。</t>
         </is>
       </c>
-      <c r="J48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2429,13 +2296,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
           <t>火线绕城三匝，没有烧到一间民屋。彤看着你，终于点头。</t>
         </is>
       </c>
-      <c r="J49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2464,14 +2329,11 @@
           <t>inkContract=1;fragments=2;karma=5</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
           <t>机关鸟只回来半只。残翼里夹着一张名单，第一行写着：无名人间。</t>
         </is>
       </c>
-      <c r="J50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2500,14 +2362,11 @@
           <t>iceLedger=1;virtue=12;karma=-6;fragments=1</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
           <t>侍童哭得很小声。他说自愿两个字，是神使替他写的。</t>
         </is>
       </c>
-      <c r="J51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2541,13 +2400,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
           <t>丹田里一半潮声，一半日火。雷云压下时，你听见九天有人翻页。</t>
         </is>
       </c>
-      <c r="J52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2576,14 +2433,11 @@
           <t>virtue=18;karma=-8;fragments=1</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
           <t>水镜没有碎。碎的是三位长老脸上的镇定。</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2612,14 +2466,11 @@
           <t>virtue=15;memory=2;fragments=1</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
           <t>剑光落下时，黄泉和碧落同时后退一步。人间第一次不在中间。</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2648,14 +2499,11 @@
           <t>karma=6;virtue=8;memory=1</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
           <t>神使说不出话。因为朱天炎狱剑上的错纹，和他腰间那把一模一样。</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2684,14 +2532,11 @@
           <t>xuanhuiBond=2;sunCinders=1;virtue=12;karma=-4</t>
         </is>
       </c>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr">
         <is>
           <t>诏书烧得很慢。玄晖看着火，像终于确认自己不是另一件法器。</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2720,14 +2565,11 @@
           <t>virtue=14;karma=-5;fragments=1</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
           <t>莫非云站在堂下，声音不高，却每个字都像白羽落在刀锋上。</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2756,14 +2598,11 @@
           <t>karma=8;fragments=2;memory=1</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
           <t>假名传出去一夜，三界各有一盏灯灭。夜哭说，鱼上钩了。</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2792,14 +2631,11 @@
           <t>virtue=20;karma=-6;fragments=1</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
           <t>有人不服，有人沉默。可城外伤者被抬进来时，所有争吵都短了一截。</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -2828,14 +2664,11 @@
           <t>memory=2;karma=10;fragments=1</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
           <t>心魔带回祭席，也带回一张和你相同的脸。你让它坐下，把灯点亮。</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2864,14 +2697,11 @@
           <t>memory=2;karma=-12</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
           <t>幽都没有惩罚你，只让你把每个被你省略的人名重新念一遍。</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2900,14 +2730,11 @@
           <t>memory=4;fragments=1;years=-99</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr">
         <is>
           <t>这一世你没赢。但下一世睁眼前，你已经听见铜门里有人开始害怕。</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2936,14 +2763,11 @@
           <t>virtue=20;memory=2</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr">
         <is>
           <t>铜门前的地面裂开，却没有吞人。黄泉和碧落第一次各退回自己的边界。</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -2972,14 +2796,11 @@
           <t>virtue=18;fragments=1;memory=2</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr">
         <is>
           <t>玄晖没有登回神座。他把最后一缕金乌火放进人间共同守着的灯里。</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -3008,14 +2829,11 @@
           <t>virtue=15;memory=3</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
       <c r="I65" t="inlineStr">
         <is>
           <t>剑光没有斩神，也没有斩鬼，只斩断那条把人间写成通路的旧线。</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -3039,11 +2857,6 @@
           <t>realmMin=5;virtueMin=90;karmaMax=45</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr"/>
-      <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
-      <c r="I66" t="inlineStr"/>
-      <c r="J66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -3077,13 +2890,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr">
         <is>
           <t>九天门开了。可门内第一张祭席，正好空着你的名字。</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -3117,13 +2928,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="H68" t="inlineStr"/>
       <c r="I68" t="inlineStr">
         <is>
           <t>十日同升，天门大开。可你分不清那是飞升，还是又一次把他献上祭席。</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -3152,14 +2961,11 @@
           <t>memory=3;fragments=1;qi=-80;years=-99</t>
         </is>
       </c>
-      <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr">
         <is>
           <t>你把胜利留给别人，把答案留给下一世。</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -3183,11 +2989,6 @@
           <t>karmaMin=65</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
-      <c r="I70" t="inlineStr"/>
-      <c r="J70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -3206,20 +3007,16 @@
           <t>death</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
           <t>memory=2;fragments=1;years=-99</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr">
         <is>
           <t>你选择下一世再来，但不是空手而来。</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -3248,14 +3045,11 @@
           <t>virtue=24;memory=3;karma=-10</t>
         </is>
       </c>
-      <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr">
         <is>
           <t>不是你一个人推开铜门。所有被当成路的人，都在这一刻向前一步。</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4386,7 +4180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4683,6 +4477,23 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>叙事规则</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>章节描述</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>章节文本只写玩家眼前所见，不提前揭示三界旧契、祭席、终局真相；高概念总结放入轮回判词。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor opening into origins and birth rolls
</commit_message>
<xml_diff>
--- a/story-config.xlsx
+++ b/story-config.xlsx
@@ -494,15 +494,15 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>八门入局</t>
+          <t>入门或远行</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>十二岁到十六岁之间，你终于被大荒某一扇门接住。
-有人递给你盾，有人递给你药杵，有人只把剑匣推到桌边，让你自己打开。
+          <t>十二岁到十六岁之间，许多门都向你开过一线。
+有人递来盾牌，有人递来药杵，也有人只把一张空白路引压在桌上。你不必立刻属于谁。
 {{status}}
-门里没有答案，只有第一条规矩。</t>
+拜入一门，是一种活法；不入诸门，也是一种活法。</t>
         </is>
       </c>
     </row>
@@ -606,7 +606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:K74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -672,6 +672,11 @@
           <t>AdvanceAct</t>
         </is>
       </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>SetOrigin</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -687,7 +692,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>greatCouncil</t>
+          <t>afterBreak</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -697,12 +702,17 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>天机营</t>
+          <t>未定</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>孩子的手印沾在天机盾背面。你还不知道他的名字，却已经知道这一世不能只顾修行。</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>西陵废墙</t>
         </is>
       </c>
     </row>
@@ -720,7 +730,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>iceHeart</t>
+          <t>afterBreak</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -730,12 +740,17 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>冰心堂</t>
+          <t>未定</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>清时把药账翻到最后一页。一个三年前死在西陵的人，被写成明日午时入炉。</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>江南药庐</t>
         </is>
       </c>
     </row>
@@ -753,7 +768,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>shadow</t>
+          <t>afterBreak</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -763,12 +778,17 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>魍魉</t>
+          <t>未定</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>夜哭没有回头，只把一枚六翼令丢进水里。令牌没有沉，反而映出你的脸。</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>雷泽沉船</t>
         </is>
       </c>
     </row>
@@ -786,7 +806,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>jadeClue</t>
+          <t>afterBreak</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -801,12 +821,17 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>云麓仙居</t>
+          <t>未定</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>星图尽头不是九天，而是一片被抹去名字的海。莫非云在页角夹了一根白羽。</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>云麓观星台</t>
         </is>
       </c>
     </row>
@@ -824,7 +849,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>tribulation</t>
+          <t>afterBreak</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -839,12 +864,17 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>弈剑听雨阁</t>
+          <t>未定</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>雨水从剑匣缝里往上流。弈剑客说：从黄泉到碧落，我只是路过人间。</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>弈剑雨亭</t>
         </is>
       </c>
     </row>
@@ -862,7 +892,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>jadeClue</t>
+          <t>afterBreak</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -877,12 +907,17 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>翎羽山庄</t>
+          <t>未定</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>遗墨把机关鸟递给你，鸟腹里滚出一粒盐晶，晶面刻着你的上一世生辰。</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>翎羽山林</t>
         </is>
       </c>
     </row>
@@ -900,7 +935,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>copperGate</t>
+          <t>afterBreak</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -910,12 +945,17 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>荒火教</t>
+          <t>未定</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>彤把长刀插进地里，问你火是用来开路，还是用来烧尽挡路的人。</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>荒火旧营</t>
         </is>
       </c>
     </row>
@@ -933,7 +973,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>foxRoad</t>
+          <t>afterBreak</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -943,12 +983,17 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>青丘客</t>
+          <t>未定</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>书生皱着眉，像是不明白自己为什么停下。火光里，九道白影一闪即逝。</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>青丘边境</t>
         </is>
       </c>
     </row>
@@ -966,7 +1011,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>northSea</t>
+          <t>afterBreak</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -981,12 +1026,17 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>北溟客</t>
+          <t>未定</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>追魂符落在雪上不燃。玄晖看了你很久，说：你认错人了，我只是路过。</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>北溟雪线</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1054,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>hell</t>
+          <t>afterBreak</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1019,12 +1069,17 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>幽都照影</t>
+          <t>未定</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>判官没有锁链，只把灯推到你面前。灯里照出的是你上一世没救走的人。</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>幽都井口</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1092,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>接过天机营残盾，把孩子手印刻进军册</t>
+          <t>拜入天机营：把残盾和军册一起接下</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1045,11 +1100,17 @@
           <t>greatCouncil</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>rootBoneMin=5</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>virtue=10;fragments=1;years=-1</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>天机营</t>
@@ -1057,9 +1118,10 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>营官说军册只记战功。你把盾背翻给他看，满厅忽然没人说话。</t>
-        </is>
-      </c>
+          <t>营官看了你的根骨，又看了盾背的孩子手印，终于把军册推到你面前。</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1070,7 +1132,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>把冰心药账翻到黑页，逼长老说出入炉二字</t>
+          <t>拜入冰心堂：从药童做起，先学救人再学用毒</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1078,11 +1140,17 @@
           <t>iceHeart</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>mindMin=4</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>iceLedger=2;virtue=8;karma=3;fragments=1</t>
-        </is>
-      </c>
+          <t>iceLedger=2;virtue=8;karma=2;fragments=1</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>冰心堂</t>
@@ -1090,9 +1158,10 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>清时的寒霜爬上账页。被写进死册的活人，正在门外排队取药。</t>
-        </is>
-      </c>
+          <t>清时把药杵递给你：手稳不稳，比灵力高不高更要紧。</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1103,7 +1172,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>接下弈剑客三剑，换他开旧阵眼</t>
+          <t>拜入弈剑听雨阁：接三剑，开旧阵眼</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1111,6 +1180,11 @@
           <t>tribulation</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>mindMin=6</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
           <t>swordHeart=2;qingyangTrace=1;qi=22;years=-1</t>
@@ -1131,6 +1205,7 @@
           <t>第三剑没有落在你身上，而是斩开雨幕。阵眼下露出四字：青阳降居。</t>
         </is>
       </c>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1141,7 +1216,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>帮云麓弟子藏起白羽，先保住莫非云证词</t>
+          <t>拜入云麓仙居：替莫非云先藏住白羽证词</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1149,11 +1224,17 @@
           <t>jadeClue</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>luckMin=4</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>moFeiyunProof=2;virtue=6;fragments=1</t>
         </is>
       </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>云麓仙居</t>
@@ -1164,6 +1245,7 @@
           <t>莫非云把白羽压在残页上。羽尖指向的不是太虚，是云麓一枚旧私印。</t>
         </is>
       </c>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1174,7 +1256,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>入太虚镜室，让邪影先照你自己的脸</t>
+          <t>拜入太虚观：入镜室，让邪影先照自己的脸</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1182,11 +1264,17 @@
           <t>heartDemon</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>mindMin=5</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
           <t>shadowTrust=1;memory=1;karma=-2</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>太虚观</t>
@@ -1197,6 +1285,7 @@
           <t>镜中邪影没有扑来，只学你的声音问：若被污名的是你，你还信门规吗？</t>
         </is>
       </c>
+      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1207,7 +1296,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>在雷泽沉船下取回六翼令，不问夜哭血脉</t>
+          <t>拜入魍魉：取回六翼令，但不问夜哭血脉</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1215,11 +1304,17 @@
           <t>shadow</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>debtMin=4</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>shadowTrust=2;karma=4;fragments=1</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>魍魉</t>
@@ -1230,6 +1325,7 @@
           <t>长老们在岸上争血统。你潜进水底，只看见令牌旁有一道替人挡刀的旧痕。</t>
         </is>
       </c>
+      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1240,7 +1336,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>替遗墨修复剑炉机关，让机关鸟飞向东海</t>
+          <t>拜入翎羽山庄：修剑炉机关，让机关鸟飞向东海</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1248,6 +1344,11 @@
           <t>jadeClue</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>luckMin=5</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
           <t>inkContract=2;fragments=1;qi=10;years=-1</t>
@@ -1268,6 +1369,7 @@
           <t>机关鸟起飞前回头看了遗墨一眼，像一个不善告别的人。</t>
         </is>
       </c>
+      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1278,7 +1380,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>陪彤劈开试锋石，拒绝放出荧惑殿里的邪靡</t>
+          <t>拜入荒火教：劈开试锋石，却不放出邪靡</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1286,11 +1388,17 @@
           <t>copperGate</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>rootBoneMin=6</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
           <t>fireOath=2;virtue=5;qi=20;karma=2</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>荒火教</t>
@@ -1301,6 +1409,7 @@
           <t>石裂三寸，地底传来笑声。彤握紧刀柄，说这把火还不到交给疯子的时候。</t>
         </is>
       </c>
+      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1311,7 +1420,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>让令狐九尾做天机编外斥候，别拆穿他的狐尾</t>
+          <t>不拜门派，只做诸门客卿：哪里缺人就往哪里去</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1319,21 +1428,28 @@
           <t>foxRoad</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>luckMin=3</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>foxBond=2;virtue=8;memory=1</t>
-        </is>
-      </c>
+          <t>wandererCred=2;virtue=8;memory=1</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
-          <t>天机营</t>
+          <t>诸门客卿</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>他把尾影藏进袖里，偏偏在妖魔冲阵时忘了藏。九道狐火照亮盾墙。</t>
-        </is>
-      </c>
+          <t>你没有接任何门帖，只收下一张空白路引。第一封信，要送去城外药棚。</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1344,131 +1460,143 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>偷读玄华名剑录残页，把剑名记进识海</t>
+          <t>做山海游侠：不入诸门，替被遗漏的人作证</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>tribulation</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>memoryMin=1</t>
-        </is>
-      </c>
+          <t>greatCouncil</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
-          <t>swordHeart=1;fragments=1;karma=2</t>
-        </is>
-      </c>
+          <t>wandererCred=3;virtue=6;karma=-2;memory=1</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
-          <t>弈剑听雨阁</t>
+          <t>山海游侠</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>残页割破手指。血落在上邪二字旁，纸页里传来黄泉水声。</t>
-        </is>
-      </c>
+          <t>八封门帖摆在桌上，你只拿走压帖的石子。石子下面，藏着一个难民写错的名字。</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>把魂灯还给清时，让他先救敌将再审情报</t>
+          <t>带着高机缘追北溟脚印，暂不定归属</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>iceHeart</t>
+          <t>northSea</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>iceLedgerMin=1</t>
+          <t>luckMin=8</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>iceLedger=1;virtue=14;karma=-4;years=-1</t>
+          <t>xuanhuiBond=1;sunCinders=1;wandererCred=1;years=-1</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>未定</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>清时没有道谢。他只是把毒针收回袖中，替敌将把断气接了回来。</t>
-        </is>
-      </c>
+          <t>雪线外有人回头看你一眼。你还没入门，却先欠下一场同行。</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>把莫非云的白羽交给冷喻，而不是交给诸门</t>
+          <t>尘债太重，先去幽都井口问清自己的死期</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>jadeClue</t>
+          <t>hell</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>moFeiyunProofMin=1</t>
+          <t>debtMin=8</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>moFeiyunProof=1;shadowTrust=1;virtue=8;karma=-3</t>
+          <t>memory=2;karma=-6;wandererCred=1</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>未定</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>冷喻没有哭。她把白羽压在旧药瓶下，瓶底云麓私印终于露出来。</t>
-        </is>
-      </c>
+          <t>井水映出四个死期，其中三个已经被人改过。</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
         <v>2</v>
       </c>
       <c r="B24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>陪令狐九尾守一夜城门，看他学会害怕</t>
+          <t>把魂灯还给清时，让他先救敌将再审情报</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>foxRoad</t>
+          <t>iceHeart</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>foxBondMin=1</t>
+          <t>iceLedgerMin=1</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>foxBond=2;virtue=10;years=-1</t>
+          <t>iceLedger=1;virtue=14;karma=-4;years=-1</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>天快亮时，他问你：若我今日怕死，还算不算懂了人间感情？</t>
+          <t>清时没有道谢。他只是把毒针收回袖中，替敌将把断气接了回来。</t>
         </is>
       </c>
     </row>
@@ -1477,26 +1605,31 @@
         <v>2</v>
       </c>
       <c r="B25" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>替玄晖把手从火里拉出来，别问他是不是神子</t>
+          <t>把莫非云的白羽交给冷喻，而不是交给诸门</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>northSea</t>
+          <t>jadeClue</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>moFeiyunProofMin=1</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>xuanhuiBond=2;sunCinders=1;virtue=5</t>
+          <t>moFeiyunProof=1;shadowTrust=1;virtue=8;karma=-3</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>火没有烧他，却把你的掌心烫出一圈残日。他低声说：神子也会冷。</t>
+          <t>冷喻没有哭。她把白羽压在旧药瓶下，瓶底云麓私印终于露出来。</t>
         </is>
       </c>
     </row>
@@ -1505,31 +1638,31 @@
         <v>2</v>
       </c>
       <c r="B26" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>与夜哭分一张暗杀名单，划掉孩子和药师的名字</t>
+          <t>陪令狐九尾守一夜城门，看他学会害怕</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>shadow</t>
+          <t>foxRoad</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>shadowTrustMin=1</t>
+          <t>foxBondMin=1</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>shadowTrust=2;virtue=6;karma=2;fragments=1</t>
+          <t>foxBond=2;virtue=10;years=-1</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>夜哭看着那两道墨痕，第一次说：影子不是谁都杀。</t>
+          <t>天快亮时，他问你：若我今日怕死，还算不算懂了人间感情？</t>
         </is>
       </c>
     </row>
@@ -1538,31 +1671,26 @@
         <v>2</v>
       </c>
       <c r="B27" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>让遗墨机关鸟带走难民，而不是追踪神域使者</t>
+          <t>替玄晖把手从火里拉出来，别问他是不是神子</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>jadeClue</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>inkContractMin=1</t>
+          <t>northSea</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>inkContract=2;virtue=12;fragments=1;years=-1</t>
+          <t>xuanhuiBond=2;sunCinders=1;virtue=5</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>机关鸟载不动所有人。遗墨拆下自己的剑炉，把第二只鸟拼到天亮。</t>
+          <t>火没有烧他，却把你的掌心烫出一圈残日。他低声说：神子也会冷。</t>
         </is>
       </c>
     </row>
@@ -1571,36 +1699,31 @@
         <v>2</v>
       </c>
       <c r="B28" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>陪彤封住荧惑殿，把邪靡的笑声锁回地底</t>
+          <t>与夜哭分一张暗杀名单，划掉孩子和药师的名字</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>copperGate</t>
+          <t>shadow</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>fireOathMin=1</t>
+          <t>shadowTrustMin=1</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>fireOath=2;virtue=8;qi=18;karma=-2</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>是</t>
+          <t>shadowTrust=2;virtue=6;karma=2;fragments=1</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>彤背对殿门站了很久。她说荒火可以输，但不能把人间交给一场疯火。</t>
+          <t>夜哭看着那两道墨痕，第一次说：影子不是谁都杀。</t>
         </is>
       </c>
     </row>
@@ -1609,31 +1732,31 @@
         <v>2</v>
       </c>
       <c r="B29" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>跟弈剑客走到黄泉渡口，问他为何总说路过</t>
+          <t>让遗墨机关鸟带走难民，而不是追踪神域使者</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>hell</t>
+          <t>jadeClue</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>swordHeartMin=2</t>
+          <t>inkContractMin=1</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>swordHeart=2;qingyangTrace=1;memory=1</t>
+          <t>inkContract=2;virtue=12;fragments=1;years=-1</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>他擦剑的手停了一下：因为停得太久，就会以为黄泉和碧落都比人间重要。</t>
+          <t>机关鸟载不动所有人。遗墨拆下自己的剑炉，把第二只鸟拼到天亮。</t>
         </is>
       </c>
     </row>
@@ -1642,31 +1765,36 @@
         <v>2</v>
       </c>
       <c r="B30" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>把冷喻旧案写进云麓星图，逼观星台亮出私印</t>
+          <t>陪彤封住荧惑殿，把邪靡的笑声锁回地底</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>greatCouncil</t>
+          <t>copperGate</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>moFeiyunProofMin=2</t>
+          <t>fireOathMin=1</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>moFeiyunProof=1;virtue=10;karma=4;fragments=1</t>
+          <t>fireOath=2;virtue=8;qi=18;karma=-2</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>是</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>星图亮起时，云麓长老先拔剑斩镜。你看见他怕的不是魔女，是证词。</t>
+          <t>彤背对殿门站了很久。她说荒火可以输，但不能把人间交给一场疯火。</t>
         </is>
       </c>
     </row>
@@ -1675,31 +1803,31 @@
         <v>2</v>
       </c>
       <c r="B31" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>在北溟雪夜听玄晖讲射日之后</t>
+          <t>跟弈剑客走到黄泉渡口，问他为何总说路过</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>northSea</t>
+          <t>hell</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>xuanhuiBondMin=2</t>
+          <t>swordHeartMin=2</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>xuanhuiBond=2;sunCinders=2;memory=1;years=-1</t>
+          <t>swordHeart=2;qingyangTrace=1;memory=1</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>他说十日坠落时，他才知道贵为神明也会被写进别人的命数。</t>
+          <t>他擦剑的手停了一下：因为停得太久，就会以为黄泉和碧落都比人间重要。</t>
         </is>
       </c>
     </row>
@@ -1708,107 +1836,97 @@
         <v>2</v>
       </c>
       <c r="B32" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>用记忆点记住所有人的名字，而不是只记线索</t>
+          <t>把冷喻旧案写进云麓星图，逼观星台亮出私印</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>death</t>
+          <t>greatCouncil</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>memoryMin=4;virtueMin=70</t>
+          <t>moFeiyunProofMin=2</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>memory=2;virtue=6;years=-99</t>
+          <t>moFeiyunProof=1;virtue=10;karma=4;fragments=1</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>这一世你没有走到铜门前。但下一世，你会更早认出他们。</t>
+          <t>星图亮起时，云麓长老先拔剑斩镜。你看见他怕的不是魔女，是证词。</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>翻开朱曦素影页，追问弈剑从何而来</t>
+          <t>在北溟雪夜听玄晖讲射日之后</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>tribulation</t>
+          <t>northSea</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>swordHeartMin=1</t>
+          <t>xuanhuiBondMin=2</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>swordHeart=1;qingyangTrace=1;qi=18</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>是</t>
+          <t>xuanhuiBond=2;sunCinders=2;memory=1;years=-1</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>创派之剑没有剑鸣，只有广成子旧印。黄帝帝师四字，被雨水泡得发白。</t>
+          <t>他说十日坠落时，他才知道贵为神明也会被写进别人的命数。</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>拓下轩辕剑残纹，查黄帝为何飞升东海</t>
+          <t>用记忆点记住所有人的名字，而不是只记线索</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>jadeClue</t>
+          <t>death</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>qingyangTraceMin=1</t>
+          <t>memoryMin=4;virtueMin=70</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>qingyangTrace=2;fragments=1;qi=12;years=-1</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>是</t>
+          <t>memory=2;virtue=6;years=-99</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>残纹尽头接着东海潮声。少昊的名字在水里一闪，像被谁故意抹去。</t>
+          <t>这一世你没有走到铜门前。但下一世，你会更早认出他们。</t>
         </is>
       </c>
     </row>
@@ -1817,31 +1935,36 @@
         <v>3</v>
       </c>
       <c r="B35" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>借天策剑立约，让天机和冰心先互认账册</t>
+          <t>翻开朱曦素影页，追问弈剑从何而来</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>greatCouncil</t>
+          <t>tribulation</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>iceLedgerMin=1</t>
+          <t>swordHeartMin=1</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>virtue=12;fragments=1;iceLedger=1</t>
+          <t>swordHeart=1;qingyangTrace=1;qi=18</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>是</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>剑没有出鞘，只横在两本册子之间。先低头的是拿军令的人。</t>
+          <t>创派之剑没有剑鸣，只有广成子旧印。黄帝帝师四字，被雨水泡得发白。</t>
         </is>
       </c>
     </row>
@@ -1850,26 +1973,36 @@
         <v>3</v>
       </c>
       <c r="B36" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>追查黑玄剑，看看玉玑子把谁写成棋子</t>
+          <t>拓下轩辕剑残纹，查黄帝为何飞升东海</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>heartDemon</t>
+          <t>jadeClue</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>qingyangTraceMin=1</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>fragments=1;karma=8;memory=1</t>
+          <t>qingyangTrace=2;fragments=1;qi=12;years=-1</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>是</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>黑玄剑影里没有狂笑，只有一张排满名字的棋盘。最边上，是你的字迹。</t>
+          <t>残纹尽头接着东海潮声。少昊的名字在水里一闪，像被谁故意抹去。</t>
         </is>
       </c>
     </row>
@@ -1878,26 +2011,31 @@
         <v>3</v>
       </c>
       <c r="B37" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>拾起上邪残锋，听见七夜离开人间那一夜</t>
+          <t>借天策剑立约，让天机和冰心先互认账册</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>hell</t>
+          <t>greatCouncil</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>iceLedgerMin=1</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>memory=1;karma=5;fragments=1</t>
+          <t>virtue=12;fragments=1;iceLedger=1</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>残锋贴近耳边时，黄泉水忽然涨潮。有人抱剑发誓，终有一日踏破九黎。</t>
+          <t>剑没有出鞘，只横在两本册子之间。先低头的是拿军令的人。</t>
         </is>
       </c>
     </row>
@@ -1906,31 +2044,26 @@
         <v>3</v>
       </c>
       <c r="B38" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>用桃木剑斩开邪影污名，不许诸门再称冷喻为天生魔女</t>
+          <t>追查黑玄剑，看看玉玑子把谁写成棋子</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>jadeClue</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>moFeiyunProofMin=2</t>
+          <t>heartDemon</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>virtue=14;shadowTrust=1;fragments=1</t>
+          <t>fragments=1;karma=8;memory=1</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>桃木剑轻得像玩具，却斩断了药瓶上的假封条。满厅没有一个人敢笑。</t>
+          <t>黑玄剑影里没有狂笑，只有一张排满名字的棋盘。最边上，是你的字迹。</t>
         </is>
       </c>
     </row>
@@ -1939,26 +2072,26 @@
         <v>3</v>
       </c>
       <c r="B39" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>读墨罂剑页，查情毒如何从云麓流进太虚</t>
+          <t>拾起上邪残锋，听见七夜离开人间那一夜</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>iceHeart</t>
+          <t>hell</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>moFeiyunProof=1;iceLedger=1;karma=3;fragments=1</t>
+          <t>memory=1;karma=5;fragments=1</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>情毒二字下压着两枚印：一枚云麓，一枚太虚。莫非云的白羽夹在中间。</t>
+          <t>残锋贴近耳边时，黄泉水忽然涨潮。有人抱剑发誓，终有一日踏破九黎。</t>
         </is>
       </c>
     </row>
@@ -1967,31 +2100,31 @@
         <v>3</v>
       </c>
       <c r="B40" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>让七星龙渊照见九天祭席，不急着拔剑</t>
+          <t>用桃木剑斩开邪影污名，不许诸门再称冷喻为天生魔女</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>ascend</t>
+          <t>jadeClue</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>swordHeartMin=3;qingyangTraceMin=2</t>
+          <t>moFeiyunProofMin=2</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>swordHeart=2;fragments=1;karma=4</t>
+          <t>virtue=14;shadowTrust=1;fragments=1</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>龙渊映出的不是神座，是一排空名。每个空名旁都放着一盏人间魂灯。</t>
+          <t>桃木剑轻得像玩具，却斩断了药瓶上的假封条。满厅没有一个人敢笑。</t>
         </is>
       </c>
     </row>
@@ -2000,36 +2133,26 @@
         <v>3</v>
       </c>
       <c r="B41" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>试铸朱天炎狱剑，确认九天神剑是否全是仿品</t>
+          <t>读墨罂剑页，查情毒如何从云麓流进太虚</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>copperGate</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>realmMin=2</t>
+          <t>iceHeart</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>qi=24;fragments=1;karma=8;years=-1</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>是</t>
+          <t>moFeiyunProof=1;iceLedger=1;karma=3;fragments=1</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>火里浮出的神纹歪了一笔。弈剑客笑了：仿得这么急，看来九天也会怕。</t>
+          <t>情毒二字下压着两枚印：一枚云麓，一枚太虚。莫非云的白羽夹在中间。</t>
         </is>
       </c>
     </row>
@@ -2038,97 +2161,102 @@
         <v>3</v>
       </c>
       <c r="B42" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>拒绝夺剑，只把名剑录抄给下一世的自己</t>
+          <t>让七星龙渊照见九天祭席，不急着拔剑</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>death</t>
+          <t>ascend</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>yearsMin=1</t>
+          <t>swordHeartMin=3;qingyangTraceMin=2</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>memory=3;swordHeart=1;fragments=1;years=-99</t>
+          <t>swordHeart=2;fragments=1;karma=4</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>你合上剑录时，听见剑匣里那第二道呼吸终于平稳下来。</t>
+          <t>龙渊映出的不是神座，是一排空名。每个空名旁都放着一盏人间魂灯。</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B43" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>把青阳痕带到东海残碑前，问少昊为何禅让颛顼</t>
+          <t>试铸朱天炎狱剑，确认九天神剑是否全是仿品</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>jadeClue</t>
+          <t>copperGate</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>qingyangTraceMin=3</t>
+          <t>realmMin=2</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>qingyangTrace=2;fragments=2;years=-1</t>
+          <t>qi=24;fragments=1;karma=8;years=-1</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>是</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>残碑没有回答，只把黄帝飞升那日的潮声还给你。</t>
+          <t>火里浮出的神纹歪了一笔。弈剑客笑了：仿得这么急，看来九天也会怕。</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B44" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>陪玄晖去幽都门前等颛顼开门</t>
+          <t>拒绝夺剑，只把名剑录抄给下一世的自己</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>hell</t>
+          <t>death</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>xuanhuiBondMin=4</t>
+          <t>yearsMin=1</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>xuanhuiBond=2;sunCinders=1;memory=1;karma=-4</t>
+          <t>memory=3;swordHeart=1;fragments=1;years=-99</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>门没有开。玄晖站到雪停，仍没有低头。你第一次觉得沉默也是一种拒绝。</t>
+          <t>你合上剑录时，听见剑匣里那第二道呼吸终于平稳下来。</t>
         </is>
       </c>
     </row>
@@ -2137,31 +2265,31 @@
         <v>4</v>
       </c>
       <c r="B45" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>把上邪残锋交给幽都判官，换轮回簿一页</t>
+          <t>把青阳痕带到东海残碑前，问少昊为何禅让颛顼</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>hell</t>
+          <t>jadeClue</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>karmaMin=25</t>
+          <t>qingyangTraceMin=3</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>memory=2;karma=-8;fragments=1</t>
+          <t>qingyangTrace=2;fragments=2;years=-1</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>判官收下残锋，却没有笑。他说黄泉不缺恨，缺的是肯认账的人。</t>
+          <t>残碑没有回答，只把黄帝飞升那日的潮声还给你。</t>
         </is>
       </c>
     </row>
@@ -2170,31 +2298,31 @@
         <v>4</v>
       </c>
       <c r="B46" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>让金乌灰落在东海潮宫，照出十日坠落的座次</t>
+          <t>陪玄晖去幽都门前等颛顼开门</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>heartDemon</t>
+          <t>hell</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>sunCindersMin=3</t>
+          <t>xuanhuiBondMin=4</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>sunCinders=2;fragments=1;karma=8</t>
+          <t>xuanhuiBond=2;sunCinders=1;memory=1;karma=-4</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>潮宫地面亮起十个空圈。玄晖只看第一个，像看一张早被烧掉的家谱。</t>
+          <t>门没有开。玄晖站到雪停，仍没有低头。你第一次觉得沉默也是一种拒绝。</t>
         </is>
       </c>
     </row>
@@ -2203,31 +2331,31 @@
         <v>4</v>
       </c>
       <c r="B47" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>请令狐九尾带青丘狐火护送凡人过雪线</t>
+          <t>把上邪残锋交给幽都判官，换轮回簿一页</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>foxRoad</t>
+          <t>hell</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>foxBondMin=2</t>
+          <t>karmaMin=25</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>foxBond=1;virtue=16;karma=-4;years=-1</t>
+          <t>memory=2;karma=-8;fragments=1</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>狐火不烫，落在孩子肩上像一小片春天。九尾却冻得脸色发白。</t>
+          <t>判官收下残锋，却没有笑。他说黄泉不缺恨，缺的是肯认账的人。</t>
         </is>
       </c>
     </row>
@@ -2236,31 +2364,31 @@
         <v>4</v>
       </c>
       <c r="B48" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>让夜哭潜入幽都边市，查谁改过你的死期</t>
+          <t>让金乌灰落在东海潮宫，照出十日坠落的座次</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>shadow</t>
+          <t>heartDemon</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>shadowTrustMin=3</t>
+          <t>sunCindersMin=3</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>shadowTrust=1;memory=2;karma=6;fragments=1</t>
+          <t>sunCinders=2;fragments=1;karma=8</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>夜哭回来时袖口结霜。他只带回一句话：你的死期，不止被改过一次。</t>
+          <t>潮宫地面亮起十个空圈。玄晖只看第一个，像看一张早被烧掉的家谱。</t>
         </is>
       </c>
     </row>
@@ -2269,36 +2397,31 @@
         <v>4</v>
       </c>
       <c r="B49" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>借荒火战阵撬开铜门外环，但先撤走城外凡人</t>
+          <t>请令狐九尾带青丘狐火护送凡人过雪线</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>copperGate</t>
+          <t>foxRoad</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>fireOathMin=2;virtueMin=60</t>
+          <t>foxBondMin=2</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>fireOath=1;qi=32;virtue=8;karma=6;fragments=1</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>是</t>
+          <t>foxBond=1;virtue=16;karma=-4;years=-1</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>火线绕城三匝，没有烧到一间民屋。彤看着你，终于点头。</t>
+          <t>狐火不烫，落在孩子肩上像一小片春天。九尾却冻得脸色发白。</t>
         </is>
       </c>
     </row>
@@ -2307,31 +2430,31 @@
         <v>4</v>
       </c>
       <c r="B50" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>让遗墨机关鸟飞入九天门缝，带回祭席名单</t>
+          <t>让夜哭潜入幽都边市，查谁改过你的死期</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>ascend</t>
+          <t>shadow</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>inkContractMin=3</t>
+          <t>shadowTrustMin=3</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>inkContract=1;fragments=2;karma=5</t>
+          <t>shadowTrust=1;memory=2;karma=6;fragments=1</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>机关鸟只回来半只。残翼里夹着一张名单，第一行写着：无名人间。</t>
+          <t>夜哭回来时袖口结霜。他只带回一句话：你的死期，不止被改过一次。</t>
         </is>
       </c>
     </row>
@@ -2340,31 +2463,36 @@
         <v>4</v>
       </c>
       <c r="B51" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>用冰心魂灯照东海侍童，问神域祭品是否自愿</t>
+          <t>借荒火战阵撬开铜门外环，但先撤走城外凡人</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>iceHeart</t>
+          <t>copperGate</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>iceLedgerMin=3;virtueMin=65</t>
+          <t>fireOathMin=2;virtueMin=60</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>iceLedger=1;virtue=12;karma=-6;fragments=1</t>
+          <t>fireOath=1;qi=32;virtue=8;karma=6;fragments=1</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>是</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>侍童哭得很小声。他说自愿两个字，是神使替他写的。</t>
+          <t>火线绕城三匝，没有烧到一间民屋。彤看着你，终于点头。</t>
         </is>
       </c>
     </row>
@@ -2373,102 +2501,102 @@
         <v>4</v>
       </c>
       <c r="B52" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>闭关炼化盐晶与残日，硬推境界去看飞升真假</t>
+          <t>让遗墨机关鸟飞入九天门缝，带回祭席名单</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>tribulation</t>
+          <t>ascend</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>realmMin=3</t>
+          <t>inkContractMin=3</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>qi=42;karma=6;years=-2</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>是</t>
+          <t>inkContract=1;fragments=2;karma=5</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>丹田里一半潮声，一半日火。雷云压下时，你听见九天有人翻页。</t>
+          <t>机关鸟只回来半只。残翼里夹着一张名单，第一行写着：无名人间。</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B53" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>把药账、白羽、六翼令一起按在水镜上</t>
+          <t>用冰心魂灯照东海侍童，问神域祭品是否自愿</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>greatCouncil</t>
+          <t>iceHeart</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>iceLedgerMin=2;moFeiyunProofMin=2;shadowTrustMin=2</t>
+          <t>iceLedgerMin=3;virtueMin=65</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>virtue=18;karma=-8;fragments=1</t>
+          <t>iceLedger=1;virtue=12;karma=-6;fragments=1</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>水镜没有碎。碎的是三位长老脸上的镇定。</t>
+          <t>侍童哭得很小声。他说自愿两个字，是神使替他写的。</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B54" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>请弈剑客以七星龙渊斩开黄泉到碧落的路影</t>
+          <t>闭关炼化盐晶与残日，硬推境界去看飞升真假</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>breakWheel</t>
+          <t>tribulation</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>swordHeartMin=5;qingyangTraceMin=4;fragmentsMin=4</t>
+          <t>realmMin=3</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>virtue=15;memory=2;fragments=1</t>
+          <t>qi=42;karma=6;years=-2</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>是</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>剑光落下时，黄泉和碧落同时后退一步。人间第一次不在中间。</t>
+          <t>丹田里一半潮声，一半日火。雷云压下时，你听见九天有人翻页。</t>
         </is>
       </c>
     </row>
@@ -2477,31 +2605,31 @@
         <v>5</v>
       </c>
       <c r="B55" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>公开九天仿剑证据，逼神使承认祭席不是荣耀</t>
+          <t>把药账、白羽、六翼令一起按在水镜上</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>ascend</t>
+          <t>greatCouncil</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>fragmentsMin=4</t>
+          <t>iceLedgerMin=2;moFeiyunProofMin=2;shadowTrustMin=2</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>karma=6;virtue=8;memory=1</t>
+          <t>virtue=18;karma=-8;fragments=1</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>神使说不出话。因为朱天炎狱剑上的错纹，和他腰间那把一模一样。</t>
+          <t>水镜没有碎。碎的是三位长老脸上的镇定。</t>
         </is>
       </c>
     </row>
@@ -2510,31 +2638,31 @@
         <v>5</v>
       </c>
       <c r="B56" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>让玄晖亲手烧掉东皇归位诏，不替他做选择</t>
+          <t>请弈剑客以七星龙渊斩开黄泉到碧落的路影</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>northSea</t>
+          <t>breakWheel</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>xuanhuiBondMin=6;sunCindersMin=5</t>
+          <t>swordHeartMin=5;qingyangTraceMin=4;fragmentsMin=4</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>xuanhuiBond=2;sunCinders=1;virtue=12;karma=-4</t>
+          <t>virtue=15;memory=2;fragments=1</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>诏书烧得很慢。玄晖看着火，像终于确认自己不是另一件法器。</t>
+          <t>剑光落下时，黄泉和碧落同时后退一步。人间第一次不在中间。</t>
         </is>
       </c>
     </row>
@@ -2543,31 +2671,31 @@
         <v>5</v>
       </c>
       <c r="B57" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>把冷喻旧案交给太虚与云麓共审，不准任何一派灭口</t>
+          <t>公开九天仿剑证据，逼神使承认祭席不是荣耀</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>greatCouncil</t>
+          <t>ascend</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>moFeiyunProofMin=3;virtueMin=60</t>
+          <t>fragmentsMin=4</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>virtue=14;karma=-5;fragments=1</t>
+          <t>karma=6;virtue=8;memory=1</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>莫非云站在堂下，声音不高，却每个字都像白羽落在刀锋上。</t>
+          <t>神使说不出话。因为朱天炎狱剑上的错纹，和他腰间那把一模一样。</t>
         </is>
       </c>
     </row>
@@ -2576,31 +2704,31 @@
         <v>5</v>
       </c>
       <c r="B58" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>用魍魉暗网散布假祭名，引出真正改簿之人</t>
+          <t>让玄晖亲手烧掉东皇归位诏，不替他做选择</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>shadow</t>
+          <t>northSea</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>shadowTrustMin=3;karmaMax=60</t>
+          <t>xuanhuiBondMin=6;sunCindersMin=5</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>karma=8;fragments=2;memory=1</t>
+          <t>xuanhuiBond=2;sunCinders=1;virtue=12;karma=-4</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>假名传出去一夜，三界各有一盏灯灭。夜哭说，鱼上钩了。</t>
+          <t>诏书烧得很慢。玄晖看着火，像终于确认自己不是另一件法器。</t>
         </is>
       </c>
     </row>
@@ -2609,11 +2737,11 @@
         <v>5</v>
       </c>
       <c r="B59" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>以天策剑重立诸门证词，先救人再问罪</t>
+          <t>把冷喻旧案交给太虚与云麓共审，不准任何一派灭口</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2623,17 +2751,17 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>virtueMin=75</t>
+          <t>moFeiyunProofMin=3;virtueMin=60</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>virtue=20;karma=-6;fragments=1</t>
+          <t>virtue=14;karma=-5;fragments=1</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>有人不服，有人沉默。可城外伤者被抬进来时，所有争吵都短了一截。</t>
+          <t>莫非云站在堂下，声音不高，却每个字都像白羽落在刀锋上。</t>
         </is>
       </c>
     </row>
@@ -2642,31 +2770,31 @@
         <v>5</v>
       </c>
       <c r="B60" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>让心魔代你入梦九天，但回来后先审自己</t>
+          <t>用魍魉暗网散布假祭名，引出真正改簿之人</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>heartDemon</t>
+          <t>shadow</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>karmaMin=35</t>
+          <t>shadowTrustMin=3;karmaMax=60</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>memory=2;karma=10;fragments=1</t>
+          <t>karma=8;fragments=2;memory=1</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>心魔带回祭席，也带回一张和你相同的脸。你让它坐下，把灯点亮。</t>
+          <t>假名传出去一夜，三界各有一盏灯灭。夜哭说，鱼上钩了。</t>
         </is>
       </c>
     </row>
@@ -2675,31 +2803,31 @@
         <v>5</v>
       </c>
       <c r="B61" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>若因果已压过道心，主动入幽都照见本心</t>
+          <t>以天策剑重立诸门证词，先救人再问罪</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>hell</t>
+          <t>greatCouncil</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>karmaMin=65</t>
+          <t>virtueMin=75</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>memory=2;karma=-12</t>
+          <t>virtue=20;karma=-6;fragments=1</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>幽都没有惩罚你，只让你把每个被你省略的人名重新念一遍。</t>
+          <t>有人不服，有人沉默。可城外伤者被抬进来时，所有争吵都短了一截。</t>
         </is>
       </c>
     </row>
@@ -2708,97 +2836,97 @@
         <v>5</v>
       </c>
       <c r="B62" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>寿元将尽，把所有证据封进轮回记忆</t>
+          <t>让心魔代你入梦九天，但回来后先审自己</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>death</t>
+          <t>heartDemon</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>yearsMin=1</t>
+          <t>karmaMin=35</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>memory=4;fragments=1;years=-99</t>
+          <t>memory=2;karma=10;fragments=1</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>这一世你没赢。但下一世睁眼前，你已经听见铜门里有人开始害怕。</t>
+          <t>心魔带回祭席，也带回一张和你相同的脸。你让它坐下，把灯点亮。</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B63" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>以诸门证词重订三界旧契：人间不是路</t>
+          <t>若因果已压过道心，主动入幽都照见本心</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>breakWheel</t>
+          <t>hell</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>fragmentsMin=6;virtueMin=80</t>
+          <t>karmaMin=65</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>virtue=20;memory=2</t>
+          <t>memory=2;karma=-12</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>铜门前的地面裂开，却没有吞人。黄泉和碧落第一次各退回自己的边界。</t>
+          <t>幽都没有惩罚你，只让你把每个被你省略的人名重新念一遍。</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B64" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>带玄晖与金乌烬上前，写下神子也有选择命运的权利</t>
+          <t>寿元将尽，把所有证据封进轮回记忆</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>breakWheel</t>
+          <t>death</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>xuanhuiBondMin=7;sunCindersMin=6;virtueMin=70</t>
+          <t>yearsMin=1</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>virtue=18;fragments=1;memory=2</t>
+          <t>memory=4;fragments=1;years=-99</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>玄晖没有登回神座。他把最后一缕金乌火放进人间共同守着的灯里。</t>
+          <t>这一世你没赢。但下一世睁眼前，你已经听见铜门里有人开始害怕。</t>
         </is>
       </c>
     </row>
@@ -2807,11 +2935,11 @@
         <v>6</v>
       </c>
       <c r="B65" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>请弈剑客出最后一剑：黄泉碧落皆路过</t>
+          <t>以诸门证词重订三界旧契：人间不是路</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2821,17 +2949,17 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>swordHeartMin=6;qingyangTraceMin=5;fragmentsMin=5</t>
+          <t>fragmentsMin=6;virtueMin=80</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>virtue=15;memory=3</t>
+          <t>virtue=20;memory=2</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>剑光没有斩神，也没有斩鬼，只斩断那条把人间写成通路的旧线。</t>
+          <t>铜门前的地面裂开，却没有吞人。黄泉和碧落第一次各退回自己的边界。</t>
         </is>
       </c>
     </row>
@@ -2840,21 +2968,31 @@
         <v>6</v>
       </c>
       <c r="B66" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>以高德行登九天，公开祭席后的旧账</t>
+          <t>带玄晖与金乌烬上前，写下神子也有选择命运的权利</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>ascend</t>
+          <t>breakWheel</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>realmMin=5;virtueMin=90;karmaMax=45</t>
+          <t>xuanhuiBondMin=7;sunCindersMin=6;virtueMin=70</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>virtue=18;fragments=1;memory=2</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>玄晖没有登回神座。他把最后一缕金乌火放进人间共同守着的灯里。</t>
         </is>
       </c>
     </row>
@@ -2863,36 +3001,31 @@
         <v>6</v>
       </c>
       <c r="B67" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>带着因果强行飞升，赌九天不敢拒你</t>
+          <t>请弈剑客出最后一剑：黄泉碧落皆路过</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>ascend</t>
+          <t>breakWheel</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>realmMin=6;karmaMin=45</t>
+          <t>swordHeartMin=6;qingyangTraceMin=5;fragmentsMin=5</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>karma=18;qi=40</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>是</t>
+          <t>virtue=15;memory=3</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>九天门开了。可门内第一张祭席，正好空着你的名字。</t>
+          <t>剑光没有斩神，也没有斩鬼，只斩断那条把人间写成通路的旧线。</t>
         </is>
       </c>
     </row>
@@ -2901,11 +3034,11 @@
         <v>6</v>
       </c>
       <c r="B68" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>强迫玄晖归位东皇，以十日之火焚开天门</t>
+          <t>以高德行登九天，公开祭席后的旧账</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2915,22 +3048,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>sunCindersMin=6;karmaMin=35</t>
-        </is>
-      </c>
-      <c r="F68" t="inlineStr">
-        <is>
-          <t>qi=60;karma=24;xuanhuiBond=-3</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>十日同升，天门大开。可你分不清那是飞升，还是又一次把他献上祭席。</t>
+          <t>realmMin=5;virtueMin=90;karmaMax=45</t>
         </is>
       </c>
     </row>
@@ -2939,31 +3057,36 @@
         <v>6</v>
       </c>
       <c r="B69" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>牺牲本世修为，换诸门凡人全数撤离</t>
+          <t>带着因果强行飞升，赌九天不敢拒你</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>death</t>
+          <t>ascend</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>virtueMin=100</t>
+          <t>realmMin=6;karmaMin=45</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>memory=3;fragments=1;qi=-80;years=-99</t>
+          <t>karma=18;qi=40</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>是</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
         <is>
-          <t>你把胜利留给别人，把答案留给下一世。</t>
+          <t>九天门开了。可门内第一张祭席，正好空着你的名字。</t>
         </is>
       </c>
     </row>
@@ -2972,21 +3095,36 @@
         <v>6</v>
       </c>
       <c r="B70" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>若因果压过道心，入幽都重走人间</t>
+          <t>强迫玄晖归位东皇，以十日之火焚开天门</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>hell</t>
+          <t>ascend</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>karmaMin=65</t>
+          <t>sunCindersMin=6;karmaMin=35</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>qi=60;karma=24;xuanhuiBond=-3</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>十日同升，天门大开。可你分不清那是飞升，还是又一次把他献上祭席。</t>
         </is>
       </c>
     </row>
@@ -2995,11 +3133,11 @@
         <v>6</v>
       </c>
       <c r="B71" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>什么都不争，只把真相刻进轮回记忆</t>
+          <t>牺牲本世修为，换诸门凡人全数撤离</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3007,14 +3145,19 @@
           <t>death</t>
         </is>
       </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>virtueMin=100</t>
+        </is>
+      </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>memory=2;fragments=1;years=-99</t>
+          <t>memory=3;fragments=1;qi=-80;years=-99</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>你选择下一世再来，但不是空手而来。</t>
+          <t>你把胜利留给别人，把答案留给下一世。</t>
         </is>
       </c>
     </row>
@@ -3023,29 +3166,80 @@
         <v>6</v>
       </c>
       <c r="B72" t="n">
+        <v>8</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>若因果压过道心，入幽都重走人间</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>hell</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>karmaMin=65</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>6</v>
+      </c>
+      <c r="B73" t="n">
+        <v>9</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>什么都不争，只把真相刻进轮回记忆</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>death</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>memory=2;fragments=1;years=-99</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>你选择下一世再来，但不是空手而来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>6</v>
+      </c>
+      <c r="B74" t="n">
         <v>10</v>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C74" t="inlineStr">
         <is>
           <t>以八门派、幽都、青丘、东海共证，结束献祭式轮回</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D74" t="inlineStr">
         <is>
           <t>breakWheel</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr">
+      <c r="E74" t="inlineStr">
         <is>
           <t>fragmentsMin=7;virtueMin=75;xuanhuiBondMin=5;swordHeartMin=4</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="F74" t="inlineStr">
         <is>
           <t>virtue=24;memory=3;karma=-10</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr">
+      <c r="I74" t="inlineStr">
         <is>
           <t>不是你一个人推开铜门。所有被当成路的人，都在这一刻向前一步。</t>
         </is>
@@ -4180,7 +4374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4494,6 +4688,40 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>开局系统</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>出生数值</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>根骨、心性、机缘、尘债由每世开局掷出，影响门派入门、游侠线、北溟/幽都特殊路线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>游侠线</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>定位</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>玩家可以不拜任何门派，成为山海游侠或诸门客卿，通过替各门派和凡人送信、作证、救人来推进主线。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Polish opening choice copy and order
</commit_message>
<xml_diff>
--- a/story-config.xlsx
+++ b/story-config.xlsx
@@ -1110,7 +1110,6 @@
           <t>virtue=10;fragments=1;years=-1</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>天机营</t>
@@ -1121,7 +1120,6 @@
           <t>营官看了你的根骨，又看了盾背的孩子手印，终于把军册推到你面前。</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1150,7 +1148,6 @@
           <t>iceLedger=2;virtue=8;karma=2;fragments=1</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>冰心堂</t>
@@ -1161,7 +1158,6 @@
           <t>清时把药杵递给你：手稳不稳，比灵力高不高更要紧。</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1205,7 +1201,6 @@
           <t>第三剑没有落在你身上，而是斩开雨幕。阵眼下露出四字：青阳降居。</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1234,7 +1229,6 @@
           <t>moFeiyunProof=2;virtue=6;fragments=1</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>云麓仙居</t>
@@ -1245,7 +1239,6 @@
           <t>莫非云把白羽压在残页上。羽尖指向的不是太虚，是云麓一枚旧私印。</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1274,7 +1267,6 @@
           <t>shadowTrust=1;memory=1;karma=-2</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>太虚观</t>
@@ -1285,7 +1277,6 @@
           <t>镜中邪影没有扑来，只学你的声音问：若被污名的是你，你还信门规吗？</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1314,7 +1305,6 @@
           <t>shadowTrust=2;karma=4;fragments=1</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>魍魉</t>
@@ -1325,7 +1315,6 @@
           <t>长老们在岸上争血统。你潜进水底，只看见令牌旁有一道替人挡刀的旧痕。</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1369,7 +1358,6 @@
           <t>机关鸟起飞前回头看了遗墨一眼，像一个不善告别的人。</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1398,7 +1386,6 @@
           <t>fireOath=2;virtue=5;qi=20;karma=2</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>荒火教</t>
@@ -1409,7 +1396,6 @@
           <t>石裂三寸，地底传来笑声。彤握紧刀柄，说这把火还不到交给疯子的时候。</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1438,7 +1424,6 @@
           <t>wandererCred=2;virtue=8;memory=1</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>诸门客卿</t>
@@ -1449,7 +1434,6 @@
           <t>你没有接任何门帖，只收下一张空白路引。第一封信，要送去城外药棚。</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1468,13 +1452,11 @@
           <t>greatCouncil</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>wandererCred=3;virtue=6;karma=-2;memory=1</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>山海游侠</t>
@@ -1485,7 +1467,6 @@
           <t>八封门帖摆在桌上，你只拿走压帖的石子。石子下面，藏着一个难民写错的名字。</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1514,7 +1495,6 @@
           <t>xuanhuiBond=1;sunCinders=1;wandererCred=1;years=-1</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>未定</t>
@@ -1525,7 +1505,6 @@
           <t>雪线外有人回头看你一眼。你还没入门，却先欠下一场同行。</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1554,7 +1533,6 @@
           <t>memory=2;karma=-6;wandererCred=1</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>未定</t>
@@ -1565,7 +1543,6 @@
           <t>井水映出四个死期，其中三个已经被人改过。</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -3307,7 +3284,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>你还没有赢得所有人的信任。有人愿意听你说一句，也有人已经把手按在剑上。</t>
+          <t>你把门令摊在掌心，也隔着灯火观察递令的人。你还站在门槛外，先看清每一条路要付出的代价。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clarify origin as story hook
</commit_message>
<xml_diff>
--- a/story-config.xlsx
+++ b/story-config.xlsx
@@ -476,7 +476,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>这一世从何处醒来</t>
+          <t>这一世缘起何处</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -494,15 +494,15 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>入门或远行</t>
+          <t>择路或远行</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>十二岁到十六岁之间，许多门都向你开过一线。
-有人递来盾牌，有人递来药杵，也有人只把一张空白路引压在桌上。你不必立刻属于谁。
+          <t>十二岁到十六岁之间，你带着那段缘起走到诸门之前。
+有人递来盾牌，有人递来药杵，也有人只把一张空白路引压在桌上。缘起只是你醒来的地方，不是要你立刻归属于谁。
 {{status}}
-拜入一门，是一种活法；不入诸门，也是一种活法。</t>
+拜入一门，是一种选择；不入诸门，也是一种选择。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update visual novel build and translations
</commit_message>
<xml_diff>
--- a/story-config.xlsx
+++ b/story-config.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CharacterLore" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ArtPools" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CharacterVisuals" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -445,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -482,7 +483,7 @@
       <c r="C2" t="inlineStr">
         <is>
           <t>你睁眼时，掌心压着一小片温热的铜锈。
-身体像刚从很深的水里浮上来。骨节发酸，心口却有一缕热意，仿佛这一世的根骨、心性、机缘和旧债正在慢慢归位。
+那东西只有指甲盖大小，边缘薄而锋利，像从某个巨大铜器上剥落下来。你握得太久，掌心被硌出一道浅红的印。
 {{status}}
 先别急着看窗外。你要先摸清这副身骨，看看它能承住多少风雨。</t>
         </is>
@@ -499,7 +500,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>十二岁到十六岁之间，你走到许多山门与营帐之前。
+          <t>你在这一世最初的几年里，走到许多山门与营帐之前。
 守门人把木牌推到你面前，药庐的童子在阶下等你回话。桌角还压着一张空白路引，墨没有干。
 {{status}}
 你不必马上归属谁。先决定今晚住在哪里。</t>
@@ -553,10 +554,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>这几夜里反复出现的方向，最后都指向北方雪线。
-你顺着风走到雪线外。雪地里有一串脚印，旁边落着不融的金灰；更远处立着一座太古铜门，门前有灯。
+          <t>雪线外的风比城中更硬。
+你跟着队伍走到最末，前面的人只让你搬药箱、扶伤者、替马车压住篷布。远处山影之间，有一道铜色的门线时隐时现，像有人把天边划开了一寸。
+没有人解释那是什么。你只知道越往北走，越多人开始沉默。
 {{status}}
-你还不知道铜门后是什么，只知道雪线不是终点。有人已经在风里等了很久。</t>
+你还没有资格靠近那道门。先看清雪地里谁在等，谁在躲，谁又把灯举得太低。</t>
         </is>
       </c>
     </row>
@@ -566,32 +568,53 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>水镜前</t>
+          <t>各自的说法</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>从雪线回来后，没有人再把雪线外的遭遇当成偶然。
-水镜被搬到厅中。灯影落在镜面上，映出的不是答案，而是每个人刚才避开过的停顿。
+          <t>从雪线回来后，没有人再把那一夜当成偶然。
+有人回军帐核名册，有人回药庐补药账，有人把剑鞘、星图、旧令和机关鸟重新放到灯下。你仍旧只是随行的人，不能替任何门派定夺，也不能替谁说完没亲眼见过的话。
 {{status}}
-这一次，不是你独自追问命运。你只能先看谁愿意开口。</t>
+先听眼前这条线上的人怎么说。你只需要分清：哪些话来自亲见，哪些话只是他们想让你相信。</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>铜门之前</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>队伍抵达太古铜门附近时，天色像被旧铜锈压住。
+长辈和守门人都在前方，你只能站在队尾，看见风从门缝里吹出，把灯火压成细线。没有人把开门的权柄交给你，但你手里留下的那些小事，终于能在此刻派上用场。
+一页名册、一盏灯、一段剑穗、一次没有说出口的犹豫，都可能让某个人少走一步死路。
+{{status}}
+这不是谁一人能扛起的命数。你能做的，只是让眼前这一刻少一个人被丢下。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
         <v>6</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>铜门之前</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>水镜没有给出答案，只把一线冷光投向北方。
-太古铜门前没有风。你听见身后有人压低呼吸，也有人把手按在兵刃、灯柄或药箱上。铜门上的锈痕一点点发热。
-你仍然不知道铜门后会有什么。可你知道，退回去的人也会被它追上。</t>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>同行之约</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>议事没有结果，夜色却已经压到廊下。
+有人要北上，有人想封门，有人只想把身边的人先带回去。你仍旧站在门外，手里拿着别人交来的名册、药灯或一封没有署名的信。
+真正的决议还在内堂，你能做的只是陪某个人多走一段，听他把没说完的话说完。
+{{status}}
+路还没有到铜门前。先照顾眼前的人。</t>
         </is>
       </c>
     </row>
@@ -606,7 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K106"/>
+  <dimension ref="A1:K149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -700,11 +723,6 @@
           <t>virtue=8;memory=1;years=-1</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>未定</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>孩子的手印留在旧盾背面。你把盾翻过来，先听见墙外有人在哭。</t>
@@ -738,11 +756,6 @@
           <t>virtue=6;iceLedger=1;years=-1</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>未定</t>
-        </is>
-      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>药炉快熄了。床边放着一张无字药签，纸角还带着血腥味。</t>
@@ -776,11 +789,6 @@
           <t>karma=3;shadowTrust=1;memory=1</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>未定</t>
-        </is>
-      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>雾里有人把半枚旧令丢进水里。令牌没有沉，只映出你的脸。</t>
@@ -819,14 +827,9 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>未定</t>
-        </is>
-      </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>星图尽头不是天，是一片被潮声擦过的黑。你捡到一根白羽。</t>
+          <t>望星台的石缝里积着海盐，星图被雨泡皱了一角。你在书页夹缝里捡到一根白羽，羽根还缠着半圈细线。</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -862,11 +865,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>未定</t>
-        </is>
-      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>雨水从亭檐往上流。柱子上刻着一句旧话，你只认得其中半句。</t>
@@ -905,11 +903,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>未定</t>
-        </is>
-      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>一只破损的机关鸟倒在树根边。鸟腹里滚出一粒盐晶，你先把它们收进袖中。</t>
@@ -948,14 +941,10 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>未定</t>
-        </is>
-      </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>试锋石裂开三寸。地底传来笑声，你把耳朵移开。</t>
+          <t>你醒在一片烧硬的黑土上，手边半埋着一块裂开的试锋石。石缝里还有余温，像有人刚把火从里面取走。
+远处营帐已经塌了，只剩几根旗杆斜在风里。你没有听见战鼓，只听见地底有一声很轻的弦响，一闪即没。</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -986,11 +975,6 @@
           <t>foxBond=1;virtue=7;memory=1</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>未定</t>
-        </is>
-      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>渡口没有船。一个书生把最后半块干粮递给孩子，又匆匆走进雾里。</t>
@@ -1024,11 +1008,6 @@
           <t>xuanhuiBond=1;sunCinders=1;virtue=4;years=-1</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>未定</t>
-        </is>
-      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>追魂符落在雪上没有燃。远处有人回头看了你一眼，又把脸藏进风里。</t>
@@ -1062,11 +1041,6 @@
           <t>memory=2;karma=-5;years=-1</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>未定</t>
-        </is>
-      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>井口没有锁链，只有一盏灯被推到你面前。灯里照出你没救走的人。</t>
@@ -1100,11 +1074,6 @@
           <t>virtue=5;wandererCred=1;memory=1</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>未定</t>
-        </is>
-      </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>渡船还没靠岸，船夫却已经知道你要过河。他问你带不带旧账。</t>
@@ -1143,11 +1112,6 @@
           <t>TRUE</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>未定</t>
-        </is>
-      </c>
       <c r="I13" t="inlineStr">
         <is>
           <t>河沙里埋着半片铜符，摸上去像晒过很久。水下有人敲了三下石头。</t>
@@ -1181,11 +1145,6 @@
           <t>luck=1;virtue=4;years=-1</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>未定</t>
-        </is>
-      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>古道两侧没有行人，只有鹿蹄印一路通向山外。你忽然不急着拜入任何山门。</t>
@@ -1219,11 +1178,6 @@
           <t>fragments=1;qingyangTrace=1;karma=1</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>未定</t>
-        </is>
-      </c>
       <c r="I15" t="inlineStr">
         <is>
           <t>潮水退去后，盐壳下露出一行旧字。海风磨平了大半，只剩一个字还清楚。</t>
@@ -1264,7 +1218,8 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>守门校尉递来一碗冷水，又把没写完的军册推到你面前。你先学会看名字，也学会看名字后面的伤。</t>
+          <t>天机营的门槛被雨水泡得发黑。守门校尉没有问你来历，只把一卷没写完的军册推到你面前，墨迹还湿着。
+天机营校尉：先别急着说自己能做什么。今夜先学会数人，少数一个，明日就少一盏灯。</t>
         </is>
       </c>
     </row>
@@ -1287,7 +1242,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>iceLedger=2;virtue=8;karma=1</t>
+          <t>iceLedger=2;virtue=8;karma=-1;qingshiBond=1</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1297,7 +1252,8 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>药庐少年把药杵放进你手里，让你先听清三个人的咳声。药炉旁没有人急着问你会不会救人。</t>
+          <t>药庐里没有人高声说话。药炉旁的少年把药杵递给你，让你先洗手，再去听最里面那张病榻上的呼吸。
+药庐少年：别急着认门规。先记住，冰心堂救人时，病人没有贵贱，也没有先后。</t>
         </is>
       </c>
     </row>
@@ -1335,7 +1291,8 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>雨亭剑客让你在雨里站到天亮。你没有拔剑，只记住雨落在鞘上的轻响。</t>
+          <t>雨亭檐下没有摆剑，只有一柄旧鞘横在石阶上。雨亭剑客没有看你的手，先让你站到檐外听雨。
+雨亭剑客：剑先不拔。站到天亮，听雨落在鞘上，也听你自己退不退。</t>
         </is>
       </c>
     </row>
@@ -1368,7 +1325,8 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>观星的人把一根白羽夹进书页里。那夜星灯没有灭，你也没有问白羽从哪里来。</t>
+          <t>云麓仙居的星灯低悬在窗前，灯芯短得几乎要熄。观星者把白羽夹进书页，袖口没有沾一点灯灰。
+观星者：今夜只守灯。它若灭了，你再问风从何处来。</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1359,8 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>镜室里积着一层灰。你扫到最后才发现，镜中的影子总比你慢半步。</t>
+          <t>太虚观的镜室灰很厚。你扫到最后，镜中的影子才慢半拍抬眼，屋里却像早有人等过很久。
+镜中影：别忙着怕我。你我今日才第一次照面，未必谁更像真的。</t>
         </is>
       </c>
     </row>
@@ -1434,7 +1393,8 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>递牌的人手很稳。夜牌入手微凉，你听见巷子深处有人把门闩放下。</t>
+          <t>旧巷的雨落不到地上，都被屋檐和斗笠接住了。递牌人把夜牌放进你掌心，木牌冰凉，却没有一点水汽。
+递牌人：收好。旧巷不怕人问，只怕人问错时候。</t>
         </is>
       </c>
     </row>
@@ -1472,7 +1432,8 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>机关师把最小的一只机关鸟推给你。鸟腹里卡着盐晶，你先学会怎样不弄断它的翅骨。</t>
+          <t>翎羽山庄的机关房里满是木屑和潮气。机关师按住机关鸟发颤的木翼，把最细的一枚铜针递给你。
+机关师：慢些。它不是死物，疼了会乱记路。</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1471,8 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>炉边女子站在火光后看你搬炭。你没有丢下木筐，她才把挡路的人拨开。</t>
+          <t>炉边女子看你把木筐搬到火旁，才让开半步。炭灰扑到你袖口，她没有替你拍掉，只把另一筐更沉的推过来。
+炉边女子：手别抖。荒火不收怕烫的人，也不收只会逞强的人。先搬炭，再谈刀。</t>
         </is>
       </c>
     </row>
@@ -1543,7 +1505,8 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>车辕上的书生把账簿丢给你。商队要过河，你先学会数车，也学会数没上车的人。</t>
+          <t>渡口的车辕陷在湿泥里，商队的人只顾数货。车辕书生把账簿抛给你，自己回头去数还没上车的人。
+车辕书生：货少一箱还能赔，人少一个，这一路就算白走。</t>
         </is>
       </c>
     </row>
@@ -1576,7 +1539,8 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>老船夫把扫帚递给你。门里的人说话很轻，杂役却常常听见最先漏出来的那一句。</t>
+          <t>老船夫把扫帚递给你，又往门内灯影里看了一眼。你第一次见他，先闻到他衣角上潮湿的江风。
+老船夫：杂役听见的事最多。听见了先放在心里，别急着拿出去换人情。</t>
         </is>
       </c>
     </row>
@@ -1604,12 +1568,13 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>iceLedger=1;virtue=12;karma=-3;years=-1</t>
+          <t>iceLedger=1;virtue=12;karma=-3;years=-1;qingshiBond=1</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>药庐少年扶着咳血的人，袖口全湿了。你没有问那人犯过什么错，只先扶住门。</t>
+          <t>后门半掩着，雨水把门槛泡得发白。药庐少年扶着一个咳血的人，袖口湿透，手却没有松。
+药庐少年：先别问他从哪里来。你按住他的腕，我听他的气。活下来的人，才有来历可问。</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1607,8 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>有人蹲在墙下，正把湿透的铃铛塞回孩子手里。你把外衣披过去。</t>
+          <t>城墙下积着一汪雨水，孩子抱着湿铃铛，铃舌已经哑了。你蹲下替他把铃绳重新系紧，才发现墙根还有几个人缩在阴影里，不敢出声。
+孩子问灯还会不会亮。你把外衣披到他肩上，只说：先跟我走，别回头看。</t>
         </is>
       </c>
     </row>
@@ -1675,7 +1641,8 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>灯灭时，墙上多出第二个人影。持刀的人没有回头，只用刀鞘敲了敲地面。</t>
+          <t>灯灭时，墙上多出第二个人影。刀鞘轻轻点地，像在量你的步子，也像在提醒你别站得太亮。
+递牌人：别站进光里。今夜看灯的人，比点灯的人多。</t>
         </is>
       </c>
     </row>
@@ -1698,7 +1665,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>pathIn=天机营|游侠</t>
+          <t>path=天机营</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1708,7 +1675,8 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>窗外有人伸手来拿军册。你按住桌沿，听见门外有人低声叹气。</t>
+          <t>窗外的手已经摸到案边，指尖带着雨水。你按住军册，也按住袖中的铜锈，听见门外有人轻轻叹了一口气。
+天机营校尉没有拔刀，只低声说：按住。账可以晚些算，册子不能在你眼前丢。</t>
         </is>
       </c>
     </row>
@@ -1741,7 +1709,8 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>机关鸟飞得歪斜，却总能避开巡夜人的灯。它把你带到一片破瓦前。</t>
+          <t>机关鸟飞得歪斜，却总能避开巡夜人的灯。它停在破瓦前，用木喙啄了三下，像在敲一扇只有它看得见的门。
+机关师：它在报路。别问它怎么知道，先看它怕什么。</t>
         </is>
       </c>
     </row>
@@ -1779,7 +1748,8 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>铜锈贴着皮肤发热。观星的人没有看你，只把书页往灯下压了压。</t>
+          <t>铜锈贴着皮肤发热，边缘硌得你腕骨发疼。观星者没有看你，只把书页往灯下压了压，不让窗外的风翻过去。
+观星者：袖口收紧些。今夜有人在找旧物，不只是在找灯。</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1787,8 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>亭中无人，剑声却从脚下传来。有人把伞留在亭外，人已经不见了。</t>
+          <t>亭中无人，剑声却从脚下传来。你没有立刻追进去，只看见门外有人把伞留给你，声音隔着雨落下。
+雨亭剑客：听到第三声就够了。再往前，是剑替你走路。</t>
         </is>
       </c>
     </row>
@@ -1840,7 +1811,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>pathIn=天机营|游侠</t>
+          <t>path=幽都旧隙</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1850,7 +1821,8 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>雨里夹着雪味。你走了很久，才看见前方有人点灯；那人没有报名字。</t>
+          <t>雨里夹着雪味，你沿着旧裂往北走了很久。风声像从地下吹上来，直到前方出现一盏没有被雨打灭的灯。
+点灯人：别站在风口。名字以后再问，先把手伸过来。</t>
         </is>
       </c>
     </row>
@@ -1883,7 +1855,8 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>有人骂你多管闲事。可火烧起来时，最先冲进巷子的也是一个你白天见过的人。</t>
+          <t>名册念到一半就停了，屋角还有几个人没有被叫到。你没有等管事回头，先把他们一个个摇醒。
+有人骂你多管闲事。可火烧起来时，最先冲进巷子的，也是白天那个被你叫醒的人。</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1889,8 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>脚步声停在床前很久。你闭着眼，听见门外的铃轻轻响了一下。</t>
+          <t>脚步声停在床前很久。你闭着眼，手却一直按着袖口的夜牌，听见门外的铃轻轻响了一下。
+那人没有进来。你也没有把看见的影子说出口。</t>
         </is>
       </c>
     </row>
@@ -1929,7 +1903,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>把无字药签浸进水里</t>
+          <t>把无字药签浸进温水里</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1944,17 +1918,13 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>fragments=1;qi=12;karma=2</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>TRUE</t>
+          <t>fragments=1;qi=8;karma=1;iceLedger=1;qingshiBond=1</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>药签背面慢慢浮出三个时辰。药庐少年看着水面，手停了一下。</t>
+          <t>无字药签浸进温水后，背面慢慢浮出三个时辰。墨色带着一点海盐味，顺着纸纹往下渗。
+药庐少年伸手拦住你：这不是药方。是有人替病人排好了谁先安静。</t>
         </is>
       </c>
     </row>
@@ -1982,12 +1952,13 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>iceLedger=2;virtue=8</t>
+          <t>moFeiyunProof=2;virtue=8</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>观星的人没有立刻接。他看着羽片上的盐痕，像在确认一件不该发生的事。</t>
+          <t>湿羽放到灯下时，盐痕一点点浮出来。观星者没有立刻接，指节却慢慢收紧。
+观星者：它不该带着海味，更不该比星图先找到你。</t>
         </is>
       </c>
     </row>
@@ -2015,12 +1986,13 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>moFeiyunProof=2;virtue=6;fragments=1</t>
+          <t>swordHeart=2;qingyangTrace=1;virtue=6;fragments=1</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>雨亭剑客把剑穗挂回墙上。它自己转了半圈，指向北边。</t>
+          <t>断剑穗被你挂回墙上，水顺着旧绳结往下滴。绳结里夹着一点黑砂，像是从很冷的河滩带回来。
+雨亭剑客看见后没有伸手扶正，只把剑架往里推了半寸。</t>
         </is>
       </c>
     </row>
@@ -2048,7 +2020,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>swordHeart=2;qingyangTrace=2;qi=10</t>
+          <t>shadowTrust=2;memory=1;qi=10</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2058,7 +2030,8 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>旧令投下的影子不止一枚。持刀的人看了一眼影子，换了握刀的手。</t>
+          <t>旧令扣在桌上，边角磨得很平，像被许多人攥过。递牌人换了握刀的手，却没有阻止你继续看。
+递牌人：别碰背面。那一面写的不是给你看的名字。</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2064,8 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>那人没有伸手接，只把刀鞘横在桌边。旧令的影子落在刀鞘上，像一条没有走完的路。</t>
+          <t>那人没有伸手接，只把刀鞘横在桌边。旧令的影子落在刀鞘上，像一条没有走完的路。
+你等他自己开口，没有替他把沉默说完。</t>
         </is>
       </c>
     </row>
@@ -2104,7 +2078,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>让机关鸟自己选择</t>
+          <t>松开机关鸟脚上的细绳</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2124,7 +2098,8 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>机关鸟啄了啄盐晶，又啄了啄你的袖口。机关师低声说：它记得路。</t>
+          <t>机关鸟啄了啄盐晶，又啄了啄你的袖口，最后把头转向风来的地方。
+机关师没有催你拆开它的腹匣，只让你松开脚上的细绳。它飞得歪，却总绕开同一片屋檐。</t>
         </is>
       </c>
     </row>
@@ -2157,7 +2132,8 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>机关鸟忽然安静下来，翅骨里的细线一根根绷直。机关师低声说：它认得这粒盐晶。</t>
+          <t>盐晶放到机关鸟旁时，木翼里的细线一根根绷直。你看见盐粒上沾着一点铜屑，像是从门缝边擦下来。
+机关师：它认得这粒盐晶。不是因为盐，是因为它被带回来过。</t>
         </is>
       </c>
     </row>
@@ -2213,7 +2189,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>xuanhuiBondMin=1</t>
+          <t>pathIn=幽都旧隙|游侠;xuanhuiBondMin=1</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2261,7 +2237,7 @@
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>车辕上的书生没有逞强。雪线外还有活人等着回家，你跟他一起绕开铜门，把人往回带。</t>
+          <t>车辕上的书生把半卷湿书塞进怀里，低声说北边的风会记住每一个太早靠近铜门的人。你没有问他的名字，只替他把车轮从雪坑里推出来。</t>
         </is>
       </c>
     </row>
@@ -2284,7 +2260,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>swordHeartMin=2</t>
+          <t>path=弈剑听雨阁;swordHeartMin=2</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -2294,7 +2270,7 @@
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>雪下传来一声轻响，像有人终于把剑放下。你第一次听见旁人叫他青阳。</t>
+          <t>雨亭剑客没有拔剑。他在雪里挖了一个很浅的坑，把断剑穗埋下，又用剑鞘压平雪面。你看见他指节发白，却没有追问。</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2303,7 @@
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>潮声从冰下传来。观星的人把白羽压在掌心，提醒你别走太快。</t>
+          <t>冰面下传来潮声，像有人在很远的地方敲门。你跟着声音走了一段，直到有人从身后喊你别再往前。</t>
         </is>
       </c>
     </row>
@@ -2340,7 +2316,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>接过校尉递来的旧盾</t>
+          <t>接过守城人递来的旧盾</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2360,7 +2336,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>盾面很冷，背后的手印却像刚留下不久。校尉把它交给你，你听见风里有人在喊。</t>
+          <t>守城人把旧盾推给你，盾沿缺了两处。他说不用你上前线，只要替后面的人挡一阵风。</t>
         </is>
       </c>
     </row>
@@ -2393,7 +2369,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>后来的人走得很慢。你没有催，只把风挡在前面，让他们一个个走过雪线。</t>
+          <t>你回身扶住落在队尾的人。雪很快盖住你们的脚印，前面的灯也因此慢了一慢。</t>
         </is>
       </c>
     </row>
@@ -2421,12 +2397,13 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>iceLedger=2;virtue=10;karma=-3</t>
+          <t>iceLedger=2;virtue=10;karma=-3;knownName=qingshi;qingshiBond=1</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>药庐少年低头很久，终于先报出自己的名字：清时。药账里另一个没写上的名字，也被他一并说出。</t>
+          <t>药庐后堂没有开审，只有几张脉案被铺在灯下。药庐少年低头很久，终于把手从药账上移开。
+药庐少年：我叫清时。账上少的不是一味药，是一个本该听见天亮的人。</t>
         </is>
       </c>
     </row>
@@ -2459,7 +2436,8 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>持刀的人没有辩解，只说自己叫夜哭。随后，他把袖中的第二枚令牌放上桌。</t>
+          <t>旧巷里没有堂审，只有一盏灯照着令牌背面。持刀的人没有坐下，只把刀鞘横在身前。
+持刀人：有些名字不是我划掉的。但我知道是谁让我递牌。</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2470,8 @@
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>观星的人把星图推到水镜前。你这才听见旁人叫他莫非云，而星图的缺口正对着东边。</t>
+          <t>星灯底下，观星的人把白羽压在潮湿的星图边。羽尖沾着一点海气，他没有让任何人先碰。
+观星者：这根羽不该带着海味。有人把它夹进星图里，又不想让我们知道它曾经沾过海水。</t>
         </is>
       </c>
     </row>
@@ -2530,7 +2509,8 @@
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>雨亭剑客说自己叫青阳，也说自己只路过人间。可他说这句话时，手一直按着剑鞘。</t>
+          <t>雨亭剑客听完众人争执，才把剑鞘轻轻放到膝上。
+雨亭剑客：剑先不拔。站到天亮，听雨落在鞘上，也听你自己退不退。</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2523,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>不审谁，先救城外的人</t>
+          <t>不等内堂争论，先救城外的人</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2563,7 +2543,8 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>水镜前少了你的声音，城外却多了几盏灯。车辕上的书生第一次没有笑。</t>
+          <t>城里还在争论，城外却已经起风。你没有等谁给一句准话，先带着杂役和商队去接还没进城的人。
+车辕上的书生第一次没有笑，只把账簿合上跟了出来。</t>
         </is>
       </c>
     </row>
@@ -2576,7 +2557,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>先看水镜里的停顿</t>
+          <t>先看每个人说话前的停顿</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2596,20 +2577,21 @@
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>你没有急着把任何东西交出去，只按住掌心那片铜锈。水镜里的影子也跟着停住，像在等你先开口。</t>
+          <t>你没有催任何人。灯影一晃，几个人同时移开目光。
+你记住的不是谁说得更像真的，而是谁在看见旧物时先摸了袖口。</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B56" t="n">
         <v>1</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>推开铜门前先回头看一眼</t>
+          <t>靠近铜门前先回头看一眼</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2629,13 +2611,13 @@
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>你回头时，看见有人终于敢在铜门前把灯举高。</t>
+          <t>你回头时，看见有人终于敢在铜门前把灯举高。你没有往前抢那一步，只把身后的人数重新数了一遍。</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B57" t="n">
         <v>2</v>
@@ -2662,20 +2644,20 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>铜锈贴上铜门缝，里面传来一声很轻的叹息。</t>
+          <t>你把那片铜锈贴近门缝。它没有发光，只在风里轻轻发热，像记起自己曾经属于这里。</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B58" t="n">
         <v>3</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>用剑鞘抵住铜门</t>
+          <t>把剑鞘递给雨亭剑客</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2695,20 +2677,20 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>剑没有出鞘。铜门却停了一息。</t>
+          <t>你把剑鞘递给雨亭剑客。他没有拔剑，只把剑鞘横在门风之前。你站在他身后，听见门缝里传来一声很轻的回响。</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B59" t="n">
         <v>4</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>独自走进铜门</t>
+          <t>独自走到铜门阴影里</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2728,13 +2710,13 @@
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>铜门后的光太亮，你听不清身后的人在喊什么。</t>
+          <t>你往前走了一步，立刻明白这不是勇气能解决的事。门内的风太旧，旧到会把一个人的名字先吹散。你停在阴影边，没有替任何人开门。</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B60" t="n">
         <v>5</v>
@@ -2756,7 +2738,7 @@
       </c>
       <c r="I60" t="inlineStr">
         <is>
-          <t>你没有打开铜门。至少这一夜，城里还有人活着。</t>
+          <t>你退后一步，先把离门最近的人拉回来。铜门没有因此关闭，但至少这一刻，没有人替所谓大义白白死去。</t>
         </is>
       </c>
     </row>
@@ -2784,12 +2766,13 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>iceLedger=2;virtue=6;karma=-1;years=-1</t>
+          <t>iceLedger=2;virtue=6;karma=-1;years=-1;qingshiBond=1</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>递针的人只说若屋里的人还在喘气，就别先问他站在哪边。</t>
+          <t>你把冷针送到药庐时，屋里只剩一盏低灯。递针的人没有解释病名，只把布包按进你手里。
+药庐少年把针排成一线，低声数着病人的呼吸。每数到第九声，窗外的雨声就像忽然远了一寸。</t>
         </is>
       </c>
     </row>
@@ -2802,7 +2785,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>把挡箭木车推到巷口</t>
+          <t>把旧木车推到巷口</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2827,7 +2810,8 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>推车的人没有说谢，只把最轻的一面木盾递给你，说别让孩子看见火光。</t>
+          <t>旧木车陷在泥里，车上堆着门板和湿草。你推了三次才把它推到巷口，正好挡住往里卷的火星。
+推车的人没有说谢，只把最轻的一块木板递给你：拿着，别让孩子看见火光。</t>
         </is>
       </c>
     </row>
@@ -2860,7 +2844,8 @@
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>隔着门有人问：如果影子不背叛人，人还会不会背叛影子？你没有立刻回答。</t>
+          <t>门内的镜光薄得像水。你没有立刻推门，只在门外停住，听见有人隔着门问你，声音却像从背后传来。
+镜中影：若影子不背叛人，人会不会先背叛影子？</t>
         </is>
       </c>
     </row>
@@ -2893,7 +2878,8 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>写信的人看见你手里的信，神色微变。他让你别拆，只替他压在星灯下面。</t>
+          <t>信封没有封口，纸角却被盐水泡过。写信的人看见你手里的信，神色微变，最后只让你替他压在星灯下面。
+他没有说收信人是谁，只说今夜风大，别让它先到。</t>
         </is>
       </c>
     </row>
@@ -2926,7 +2912,8 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>机关师接过机关鸟，先检查它有没有受惊，再问你盐晶是从哪里滚出来的。</t>
+          <t>机关师接过机关鸟，先检查它有没有受惊，再问你盐晶是从哪里滚出来的。他问得很慢，像怕再碰断木翼里那根细线。
+你没有急着回答，只把匣子推到他手边。</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2946,8 @@
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>镜室里的人没有擦镜，只在灰上添了一笔。镜中的影子忽然安静下来。</t>
+          <t>镜室里的人没有擦镜，只在灰上添了一笔。镜中的影子忽然安静下来，像终于等到有人把话说到它能听懂的位置。
+你没有问它是不是人，只问它昨夜看见了什么。</t>
         </is>
       </c>
     </row>
@@ -2987,12 +2975,13 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>iceLedger=3;virtue=8;karma=-2</t>
+          <t>iceLedger=3;virtue=8;karma=-2;qingshiBond=1</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>一个人看时辰，一个人看药味。两人谁也没先说话，却同时把药炉挪近了些。</t>
+          <t>你没有让一个人单独拿走药签。一个人看时辰，一个人闻药味，谁也没有先下结论。
+炉火一亮，纸背上的潮痕终于停住。药庐少年把那页夹进账里，写下：先救仍会发声的人。</t>
         </is>
       </c>
     </row>
@@ -3015,7 +3004,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>pathIn=天机营|荒火营地|游侠</t>
+          <t>path=天机营</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -3025,7 +3014,8 @@
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>校尉用指节碰了碰铜锈边缘，说这种痕迹不像战场留下的，更像有人曾经想把门重新合上。</t>
+          <t>你把铜锈放到军册旁。校尉没有伸手拿，只用指节碰了碰边缘，像怕它烫到掌心。
+他看了很久才说：这不像战场留下的痕迹，更像有人曾经想把门重新合上。</t>
         </is>
       </c>
     </row>
@@ -3048,7 +3038,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>xuanhuiBondMin=2</t>
+          <t>pathIn=幽都旧隙|游侠;xuanhuiBondMin=2</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -3129,7 +3119,8 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>雨亭剑客说完那句旧话就闭了嘴。雪落在剑鞘上，没有化。</t>
+          <t>风雪落在剑鞘上，没有立刻化开。雨亭剑客说完那句旧话就闭了嘴，像把后半句留给了路。
+你没有催他，只记住他看向北方时，眼里没有胜意。</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3153,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>白羽落在冰面上，指向潮声更深的地方。观星的人没有回头，只抬手让你慢些。</t>
+          <t>白羽落在冰面上，被风推着滑出很短一截，停在潮声更重的地方。观星的人没有回头，只抬手让你慢些。</t>
         </is>
       </c>
     </row>
@@ -3185,17 +3176,17 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>path=冰心堂;iceLedgerMin=3</t>
+          <t>path=冰心堂;iceLedgerMin=3;knownName=qingshi</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>iceLedger=3;virtue=10;karma=-3</t>
+          <t>iceLedger=3;virtue=10;karma=-3;qingshiBond=1</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>另一个药庐弟子接过笔。清时第一次没有抢话，药账上终于多出一个活人的名字。</t>
+          <t>另一个药庐弟子接过笔，先写病人的名字，再写药量。清时第一次没有抢话，只在旁边添了一行小字：潮声入肺，灯火不可断。</t>
         </is>
       </c>
     </row>
@@ -3228,7 +3219,8 @@
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>军册和商队账簿对不上。你没有急着问责，而是沿着缺口又找回三个被漏掉的人。</t>
+          <t>城门名册和商队账簿对不上。你没有急着问责，而是沿着缺口又找回三个被漏掉的人。
+有人说这只是小误差。你把账簿翻到空白处：人命不该叫误差。</t>
         </is>
       </c>
     </row>
@@ -3261,7 +3253,8 @@
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>镜里的人没有急着辩解，镜外的人也没有立刻退开。两句话落下后，水镜里的影子终于稳了一寸。</t>
+          <t>镜里的人没有急着辩解，镜外的人也没有立刻退开。两句话落下后，水镜里的影子稳了一寸。
+你没有判断谁赢了，只记住谁说话时避开了镜面。</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3277,7 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>path=魍魉;shadowTrustMin=3</t>
+          <t>path=魍魉;shadowTrustMin=3;knownName=yeku</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3327,13 +3320,14 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>机关师拆得很慢，像怕弄疼那只鸟。盐晶里落出一粒细小的铜屑，你第一次听见有人叫他遗墨。</t>
+          <t>机关师拆得很慢，像怕弄疼那只鸟。盐晶里落出一粒细小的铜屑，你第一次听见有人叫他遗墨。
+遗墨没有抬头：它飞过的地方，不该有铜门的气味。</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B78" t="n">
         <v>6</v>
@@ -3366,7 +3360,7 @@
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B79" t="n">
         <v>7</v>
@@ -3399,7 +3393,7 @@
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B80" t="n">
         <v>8</v>
@@ -3432,7 +3426,7 @@
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B81" t="n">
         <v>9</v>
@@ -3449,7 +3443,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>pathIn=天机营|游侠;xuanhuiBondMin=4</t>
+          <t>pathIn=幽都旧隙|游侠;xuanhuiBondMin=4</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3492,7 +3486,8 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>校尉把缺页摊在灯下，只让你先数伤号，不许先数功劳。</t>
+          <t>缺页边缘被雨泡卷，像是有人匆忙从册中撕走。校尉用刀鞘压住最上面的名字，没有让旁人靠近。
+天机营校尉：先数伤号。功劳迟一夜不会死，人会。</t>
         </is>
       </c>
     </row>
@@ -3520,12 +3515,13 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>xuanhuiBond=1;virtue=5;years=-1</t>
+          <t>virtue=5;memory=1;years=-1</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
         <is>
-          <t>北墙的风里夹着雪味。你把灯重新挂好，看见墙外有一行很浅的脚印。</t>
+          <t>北墙的巡灯被雨打得只剩一层薄光。你踮脚把灯重新挂好，才看见墙外的脚印被雨水冲散。
+天机营校尉按住你的肩：别喊。先记人数，再看脚印。守城的人，不能被风牵着跑。</t>
         </is>
       </c>
     </row>
@@ -3596,7 +3592,8 @@
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>门外有人低声说只是借一副弩机。你没有开门，只把门闩又推紧了一寸。</t>
+          <t>军械库外有人低声说只是借一副弩机，明早就还。你没有答话，只把门闩又推紧一寸，听见里面的弦机轻轻震了一下。
+守门人看了你一眼：有些门开一次，后面死的人就不止一个。</t>
         </is>
       </c>
     </row>
@@ -3662,7 +3659,8 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>校尉看完名册，先把刀放下。他说这不是军功簿，是活人簿。</t>
+          <t>你把伤号名册推到校尉面前。屋里的人本想先问缺页，他却先把刀放下，一行一行把还活着的人圈出来。
+天机营校尉：这不是军功簿，是活人簿。谁把人命记成功劳，我先问谁。</t>
         </is>
       </c>
     </row>
@@ -3690,12 +3688,13 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>xuanhuiBond=1;sunCinders=1;fragments=1</t>
+          <t>virtue=8;wandererCred=1;fragments=1</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>巡灯图贴上墙时，最北边那一点墨迹慢慢渗开，像雪里有人回头。</t>
+          <t>巡灯图贴上墙时，几处缺口同时显出来。校尉没有解释，只让你把伤号棚、军械库和北墙的灯位重新连成一线。
+他低声说：下次风从那里来，先护人，再追影。</t>
         </is>
       </c>
     </row>
@@ -3733,7 +3732,8 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>你没有追进雨里，只在檐下听完三声剑响。第三声落下时，剑鞘上的水珠往北滚了一寸。</t>
+          <t>你没有追进雨里，只在檐下听完三声剑响。第三声落下时，剑鞘上的水珠往北滚了一寸。
+雨亭剑客从雨外看你：能停住，比能追上更难。</t>
         </is>
       </c>
     </row>
@@ -3766,7 +3766,8 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>剑架上的旧痕被你一点点擦出来。有人经过门外，没有进来，只留下一句：别让剑先替你选路。</t>
+          <t>剑架上的雨水顺着旧痕往下流。你一点点擦出来，才发现那些痕迹不是新伤，而像多年前有人把剑放回去时压出的印。
+雨亭剑客：别让剑先替你选路。它选得太快，人会跟不上。</t>
         </is>
       </c>
     </row>
@@ -3804,7 +3805,8 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>细线缠得很紧，你拆到最后才看见里面还夹着一粒潮湿盐晶。机关师让你先别声张。</t>
+          <t>细线缠得很紧，你拆到最后才看见里面还夹着一粒潮湿盐晶。机关师忽然按住你的手，没有让那粒盐晶滚到灯下。
+机关师：先别声张。它不是自己飞到这里来的。</t>
         </is>
       </c>
     </row>
@@ -3837,7 +3839,8 @@
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>木翼边缘有被火燎过的黑痕。你把它收进匣里，听见匣底轻轻响了一声。</t>
+          <t>木翼边缘有被火燎过的黑痕。你把它收进匣里，听见匣底轻轻响了一声，像还有什么东西不肯安静。
+机关师没有打开匣子，只让你记住那一声响。</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3873,8 @@
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>短芯亮起来时，书页里的白羽没有动，窗外的云却往低处压了压。</t>
+          <t>你剪短灯芯，火光稳了一点。书页里的白羽没有动，羽根那半圈细线却被照得发亮。
+观星者让你别抬头：天上的说法太远，先看灯下是谁动过这页纸。</t>
         </is>
       </c>
     </row>
@@ -3903,7 +3907,8 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>星图上没有墨迹，纸背却有盐水干过的皱痕。观星的人让你明日再看。</t>
+          <t>星图上没有墨迹，纸背却有盐水干过的皱痕。你把它压回书页，指尖摸到一道细得像羽轴的折痕。
+观星的人让你明日再看：现在看，只会把自己也折进去。</t>
         </is>
       </c>
     </row>
@@ -3931,12 +3936,13 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>iceLedger=1;virtue=6</t>
+          <t>iceLedger=1;virtue=6;qingshiBond=1</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>水热起来以前，后门的咳声又轻了一点。童子低声说，今晚不能只看药方。</t>
+          <t>炉边的水凉了，药气沉在碗底。你重新添火，火星一起，病榻上那口被雨声压住的气终于续了半寸。
+药童看着水面：今晚的病不只在身上。潮气进了药里，也进了人的梦里。</t>
         </is>
       </c>
     </row>
@@ -3964,12 +3970,13 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>iceLedger=1;memory=1;karma=-1</t>
+          <t>iceLedger=1;memory=1;karma=-1;qingshiBond=1</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>你把三次咳声记在纸角。药童看了很久，说这不是同一种病。</t>
+          <t>你把三次咳声记在纸角：第一声急，第二声短，第三声像被水堵住。药童看了很久，才把药杵放下。
+药庐少年：不是同一种病。有人把潮声和死期，一起揉进了一口药里。</t>
         </is>
       </c>
     </row>
@@ -4002,7 +4009,8 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>灰被擦开后，镜中多出一道很淡的门缝。你没有伸手去碰。</t>
+          <t>灰被擦开后，镜中多出一道很淡的门缝。你没有伸手去碰，只看见自己的影子先一步往后退。
+门缝很快消失，镜脚旁却留下了一点湿痕。</t>
         </is>
       </c>
     </row>
@@ -4040,13 +4048,14 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>夜牌贴着袖口发凉。巷口有人走过，你听见他故意踩碎了一片瓦。</t>
+          <t>夜牌贴着袖口发凉。巷口有人走过，故意踩碎了一片瓦，让你知道他来过，也让别人以为他走远了。
+你把牌藏得更深，记住那人左脚落地比右脚轻半拍。</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B99" t="n">
         <v>4.5</v>
@@ -4068,7 +4077,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>你没有推开铜门，也没有离开。风从铜门缝里吹出来，你把最近的一盏灯护到天亮。</t>
+          <t>你在铜门前多守了一夜。没有奇迹发生，只有几个原本想冲进去的人，在天亮前终于冷静下来。</t>
         </is>
       </c>
     </row>
@@ -4096,12 +4105,13 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>iceLedger=1;virtue=6;years=-1</t>
+          <t>iceLedger=1;virtue=6;years=-1;qingshiBond=1</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>药箱压得肩头发疼。你没问雪线后有什么，只先确认药瓶没有碎。</t>
+          <t>药箱压得肩头发疼，箱底的铜铃一路不响。药庐少年走在你身侧，每隔十步就停下来听一次风里有没有咳声。
+他没有解释海寂是什么，只说若一个人连咳都咳不出，才最该被听见。</t>
         </is>
       </c>
     </row>
@@ -4300,6 +4310,1455 @@
       <c r="I106" t="inlineStr">
         <is>
           <t>炉灰落在雪上，很快被风吹浅。你还是一段段标下去，至少后来的人知道该往哪边退。</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>6</v>
+      </c>
+      <c r="B107" t="n">
+        <v>1</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>随玄晖去雪线外看灯</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>pathIn=幽都旧隙|游侠;knownName=xuanhui;xuanhuiBondMin=3</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>xuanhuiBond=2;sunCinders=1;virtue=6;years=-1</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>玄晖把灯递到你手里，却没有松开。
+玄晖：别急着问我的名字。灯在这里不是照给我看的。你若想把人带回去，就先看清它照不到哪里。</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>6</v>
+      </c>
+      <c r="B108" t="n">
+        <v>2</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>随青阳走一段雨后的路</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>path=弈剑听雨阁;knownName=qingyang;swordHeartMin=3</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>swordHeart=2;qingyangTrace=1;qi=12;years=-1</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>雨停后，青阳走得很慢。他没有说自己来自哪里，只问你昨夜埋下的剑穗有没有被雪盖住。
+雨水沿着剑鞘往下落，落到石阶尽头时，声音忽然变得很远。你没有追问那声音通向哪里，只跟着他把这段路走完。</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>6</v>
+      </c>
+      <c r="B109" t="n">
+        <v>3</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>随莫非云去听冰下潮声</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>path=云麓仙居;knownName=moFeiyun;moFeiyunProofMin=3</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>moFeiyunProof=2;fragments=1;memory=1;years=-1</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>莫非云没有抬头看星，只带你去听冰下的潮声。
+莫非云：星图不是命令。它只是提醒我们，哪一处沉默太久。</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>6</v>
+      </c>
+      <c r="B110" t="n">
+        <v>4</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>陪清时守完最后一页药账</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>path=冰心堂;knownName=qingshi;iceLedgerMin=4</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>iceLedger=2;virtue=10;karma=-3;years=-1;qingshiBond=2</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>清时把最后一页药账推到你面前，墨迹还没干。屋外有人催你们动身，他却先把病榻旁的灯一盏盏添满。
+清时：我不是要你替我翻案。我只想知道，下一次潮声压住人的气息时，我们能不能早一点听见。</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>6</v>
+      </c>
+      <c r="B111" t="n">
+        <v>5</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>随夜哭走进旧巷深处</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>path=魍魉;knownName=yeku;shadowTrustMin=4</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>shadowTrust=2;fragments=1;karma=-1;years=-1</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>夜哭把第二枚令牌别回袖中，巷子里只剩一盏很低的灯。他走在前面，却始终没有让你的影子落到他脚下。
+夜哭：跟我走可以，但别把影子交给我。旧巷最怕有人把活人当成暗号。</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>6</v>
+      </c>
+      <c r="B112" t="n">
+        <v>6</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>跟遗墨把机关鸟放回风里</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>path=翎羽山庄;knownName=yimo;inkContractMin=4</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>inkContract=2;virtue=6;memory=1;years=-1</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>遗墨没有立刻放手，只把机关鸟腹中的盐晶重新扣好。木翼微微一振，先试探风向，再偏向北方。
+遗墨：它不是在替我们找路。它只是记得哪里曾经疼过。</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>6</v>
+      </c>
+      <c r="B113" t="n">
+        <v>20</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>不跟任何人走，先独自理清来路</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>memory=2;virtue=3;years=-1</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>你没有跟任何人离开。廊下的灯一盏盏暗下去，你把听见的名字和没听懂的沉默分成两边，免得自己太早替谁下结论。</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>7</v>
+      </c>
+      <c r="B114" t="n">
+        <v>10</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>跟玄晖把灯举到铜门外</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>xuanhuiEnding</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>pathIn=幽都旧隙|游侠;knownName=xuanhui;xuanhuiBondMin=5</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>sunCinders=1;virtue=10;memory=2</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>玄晖没有跨进铜门，只把灯举到门外。你站在他身侧，看见雪线后的路一点点亮起来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>7</v>
+      </c>
+      <c r="B115" t="n">
+        <v>11</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>跟青阳绕过铜门侧影</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>qingyangEnding</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>path=弈剑听雨阁;knownName=qingyang;swordHeartMin=5</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>qingyangTrace=2;virtue=8;memory=2</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>青阳把剑鞘压低，没有让剑替你们开路。你们沿铜门侧影走过去，雨声一直没有停。</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>7</v>
+      </c>
+      <c r="B116" t="n">
+        <v>12</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>跟莫非云去看东海潮声</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>mofeiyunEnding</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>path=云麓仙居;knownName=moFeiyun;moFeiyunProofMin=5</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>fragments=1;memory=2;virtue=6</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>莫非云把白羽贴在水镜边缘。镜面没有碎，只把潮声送到铜门前。</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>6</v>
+      </c>
+      <c r="B117" t="n">
+        <v>21</v>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>先问身边人愿不愿回头</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>virtue=5;memory=1;years=-1</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>你没有催队伍北上，只先问离你最近的人要不要回头。那人怔了一下，像终于被允许承认自己害怕。</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>6</v>
+      </c>
+      <c r="B118" t="n">
+        <v>22</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>把灯留给最慢的人</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>virtue=7;karma=-1;years=-1</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>你把灯留给走得最慢的人。前面的人因此等了一会儿，没人称赞你，但也没人再催他快些。</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>2</v>
+      </c>
+      <c r="B119" t="n">
+        <v>30</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>守住圣火殿前的火盆</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>path=荒火营地</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>fireOath=2;virtue=6;years=-1</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>雨水顺着檐角落进火盆，火苗却只是低了一低。你用衣袖替它挡住斜雨，才看见盆沿刻着许多被磨平的名字。
+炉边女子把干炭递给你：记住，圣火先照活人，再照兵刃。荒火若只会烧，九黎早就被自己烧空了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>2</v>
+      </c>
+      <c r="B120" t="n">
+        <v>31</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>去试锋石下听裂纹</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>path=荒火营地</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>fireOath=2;fragments=1;karma=1</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>你跪到试锋石旁，把耳朵贴近那道新裂。石中没有战鼓，只有一声被火烤紧的细弦，断断续续，像有人在很远处试音。
+炉边女子的脸色沉下去。她没有解释，只把你的手从石上拉开：这声音先别告诉旁人，尤其别告诉想借火立功的人。</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>3</v>
+      </c>
+      <c r="B121" t="n">
+        <v>30</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>把试锋石旁的灰纹描下来</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>path=荒火营地;fireOathMin=2</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>fireOath=2;fragments=1;virtue=4</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>你用炭条沿着石旁灰纹描了一遍。那些纹路起初像刀痕，描到末尾才连成一段折回的曲谱；最末两个字，被火熏得发黑，却还认得出是“乐风”。
+炉边女子看了很久，才低声说：祝融传火，不是为了让人学会恨水。你若真听见弦音，先记住它救过谁。</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>3</v>
+      </c>
+      <c r="B122" t="n">
+        <v>31</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>把炭车推回圣火殿侧门</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>path=荒火营地</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>fireOath=1;virtue=8;years=-1</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>炭车卡在侧门外的泥里，你推到肩背发麻，门内才有人把闩打开。热浪卷出来，里面没有兵器，只有一排排被火烘干的旧衣和伤者的鞋。
+炉边女子：先让撤回来的人有衣穿。荒火若只剩威风，就不配叫圣火。</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>4</v>
+      </c>
+      <c r="B123" t="n">
+        <v>30</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>沿圣火暗纹走进熔岩旧殿</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>path=荒火营地;fireOathMin=3</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>fireOath=3;changqinEcho=1;memory=1;years=-1</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>你顺着火盆底下延出的暗纹往殿后走。石阶越往下越热，却没有战鼓声，只有那段细弦越来越清楚。
+旧殿壁上刻着残缺的图：有人从倾塌的山影里拾起余焰，又把暴烈的火兽镇回山下。炉边女子站在你身后，低声说荒火守这处旧殿，不是为了把怒气养大。你这才把手从刀柄上松开。</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>5</v>
+      </c>
+      <c r="B124" t="n">
+        <v>30</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>请炉边女子说出琴声来历</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>path=荒火营地;changqinEchoMin=1</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>changqinEcho=2;fireOath=1;virtue=6</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>你把描下来的灰纹放到炉边女子面前。她没有立刻回答，只把刀放在膝上，像是先压住自己心里的旧火。
+炉边女子：那不是凡琴。相传祝融有子，名太子长琴，抱琴而生，始作乐风。不周山一役后，荒火山里只剩一点残响。我们守它，不是为了请神复仇。</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>6</v>
+      </c>
+      <c r="B125" t="n">
+        <v>30</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>随炉边女子去听圣火里的残响</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>path=荒火营地;knownName=changqin;changqinEchoMin=2</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>changqinEcho=2;fireOath=1;virtue=8;years=-1</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>夜深后，炉边女子带你绕到圣火殿后。火被压得很低，弦音反而清楚；你没有看见神祇，只看见火里有一道影子俯身按住断弦。
+炉边女子：别把他当成来替我们复仇的神。若太子长琴还剩一缕声息，也该先问人间还疼不疼。</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>7</v>
+      </c>
+      <c r="B126" t="n">
+        <v>30</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>把乐风留在铜门外</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>changqinEnding</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>path=荒火营地;knownName=changqin;changqinEchoMin=4;fireOathMin=5</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>virtue=12;memory=2;fragments=1</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>铜门前的风把火光压得很低。你没有让圣火去烧门，只把那段乐风留在门外，让它先照见退回来的人，再照见门上的裂纹。
+炉边女子站在你身后，第一次没有催你往前。火光向后退了一步，九黎山下那些仍在守夜的人，也因此没有被铜门吞进光里。</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>1</v>
+      </c>
+      <c r="B127" t="n">
+        <v>90</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>沿北边雪味去寻灯</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>xuanhuiBond=2;sunCinders=1;virtue=4;years=-1</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>幽都旧隙</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>你没有进任何山门，只沿着雨里的雪味往北走。城外有一道旧裂，裂口里没有鬼哭，只有一盏灯在很远处亮着。
+点灯人：别站在风口。名字以后再问，先把手伸过来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>2</v>
+      </c>
+      <c r="B128" t="n">
+        <v>40</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>收起北墙外落下的竹筒</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>path=天机营</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>qiyeTrace=1;virtue=5;years=-1</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>巡灯刚补上，墙外雪线里滚来一只裂开的竹筒。你没有追出去，只用盾沿压住它，等校尉把火遮严。
+竹筒里没有姓名，只有七道浅刻。校尉看完后把它扣进军册：朔方来的军令，最先找的从来不是城门，是井口、粮仓和人心。</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>4</v>
+      </c>
+      <c r="B129" t="n">
+        <v>40</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>守住撤民小路的灯</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>path=天机营;qiyeTraceMin=2</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>qiyeTrace=2;virtue=10;years=-1</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>第三夜，北墙外没有鼓声，只有黑甲贴着雪雾往前压。城里有孩子哭，也有人想把撤民小路上的灯先灭掉，免得被敌军看见。
+你让弩机暂缓，先把灯罩转向城内。灯光不再照路口，却照见每一个正在撤离的人。墙外的黑甲停了一息，像是也看懂了这座城先护谁。</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>5</v>
+      </c>
+      <c r="B130" t="n">
+        <v>40</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>翻出朔方旧卷</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>path=天机营;qiyeTraceMin=4</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>qiyeTrace=2;virtue=5;memory=1</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>雨停后，校尉从军册夹层里取出一页旧卷。卷上写着朔方旧帅七夜，也写着几处旧战场的退路。
+校尉没有把旧卷交给你，只让你站在灯下帮他看清缺损的字：知道对面是谁，不是为了恨得更响，是为了别被他的名声吓乱阵脚。</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>6</v>
+      </c>
+      <c r="B131" t="n">
+        <v>40</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>把上邪剑页夹回军册</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>path=天机营;qiyeTraceMin=5</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>qiyeTrace=2;virtue=6;karma=-1;memory=1</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>水镜边压着一页《玄华名剑录》的残抄。纸角被火燎过，仍能辨出一行字：上邪剑，眷夫人以命祭剑，武观（七夜）佩剑，离恨之剑。
+你没有把这页残抄传出去。一个人的旧名解释不了今夜的刀兵，却能提醒你：城外那道军令也曾从人间来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>7</v>
+      </c>
+      <c r="B132" t="n">
+        <v>40</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>把朔方军路呈给校尉</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>qiyeEnding</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>path=天机营;knownName=wuguan;qiyeTraceMin=7</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>virtue=12;memory=2;fragments=1</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>铜门前，你把七道刻痕、撤民小路和上邪残页呈给天机营校尉。你不是求和，也不是投降，只是把你见过的路、人数和伤口一一说清。
+墙外许久没有传令。那一夜，北墙没有破，井口没有毒，撤民的小路也没有断。</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>3</v>
+      </c>
+      <c r="B133" t="n">
+        <v>40</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>把七道刻痕抄进军册</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>path=天机营;qiyeTraceMin=1</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>qiyeTrace=2;virtue=6;fragments=1</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>你把竹筒上的七道刻痕一笔一笔抄进军册，才发现它们对应的不是攻城顺序，而是城中最容易断掉的地方：水井、药棚、伤号棚、粮车、弩台、旧巷和北墙角门。
+校尉低声说：对面的人熟悉守城，也熟悉人会在什么时候害怕。先别问他是谁，把这些地方守住。</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>1</v>
+      </c>
+      <c r="B134" t="n">
+        <v>95</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>在山门前停住，先认出这阵风</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>lifeMin=2;memoryMin=5</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>memory=2;fragments=1;virtue=3</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>游侠</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>你没有立刻走向任何山门。风从阶下吹过来，带着一点上一世也闻过的灰味。
+这一次，你先记住风从哪里来，再决定今晚住在哪里。</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>3</v>
+      </c>
+      <c r="B135" t="n">
+        <v>80</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>把铜锈贴在桌角旧痕上</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>lifeMin=3;memoryMin=8;fragmentsMin=2</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>memory=2;fragments=1;karma=-1</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>你把铜锈贴到桌角那道浅痕上。断口刚好压住木纹里一处凹陷，像这张桌子曾被同样的东西硌过很多次。
+旁人还在争吵，你没有打断他们，只把桌角、铜锈和掌心的红印一起记下来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>5</v>
+      </c>
+      <c r="B136" t="n">
+        <v>80</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>不急着看众人，先看旧物下方的水痕</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>lifeMin=4;memoryMin=11;fragmentsMin=3</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>memory=2;fragments=1;virtue=4</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>众人都盯着各自带回的旧物时，你退后半步，看见桌面边缘有一道反复干湿过的水痕。
+那道水痕不属于今夜。它从桌角绕到东侧，干了又湿，湿了又干，像每一次有人搬动旧物时都刻意避开那里。你没有立刻声张，只记住水痕停住的方向。</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>6</v>
+      </c>
+      <c r="B137" t="n">
+        <v>80</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>把几条旧路的方向并在一起</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>lifeMin=5;memoryMin=14;fragmentsMin=4</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>memory=2;fragments=1;virtue=5;years=-1</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>你把雪灯、白羽、旧令、试锋石灰纹和军册缺页分开放在地上。
+它们并不属于同一个人，也没有给出同一个答案。你只看见一件事：每当有人被逼着在开门和救人之间选边，铜锈就会先热起来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>7</v>
+      </c>
+      <c r="B138" t="n">
+        <v>80</v>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>把这一世记错的地方说给潮声听</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>eastSeaSecretEnding</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>lifeMin=6;memoryMin=18;fragmentsMin=6;virtueMin=70</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>memory=3;fragments=1;virtue=8</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>你没有往铜门前抢那一步。你只是转向东海来的风，把所有轮回里反复错位的细节，一处一处说出来。</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>2</v>
+      </c>
+      <c r="B139" t="n">
+        <v>80</v>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>摸清铜锈边缘的断口</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>memoryMin=2</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>copperInsight=1;memory=1</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>你把掌心那片铜锈翻到灯下，才发现它不是铜钱，也不像兵器碎片。
+它的一侧粗糙，像从很大的铸物上剥落；另一侧却被磨得很平，仿佛曾被很多人反复按住。</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>3</v>
+      </c>
+      <c r="B140" t="n">
+        <v>82</v>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>把铜锈放在灯下慢慢转动</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>copperInsightMin=1</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>copperInsight=1;memory=1</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>铜锈在灯下转过半圈，绿锈里浮出一点黑金色的旧痕。
+那道旧痕卡在断口边，像门合上时被夹过，又像后来有人用掌心反复把它按回原处。</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>5</v>
+      </c>
+      <c r="B141" t="n">
+        <v>82</v>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>只看铜锈背面那一点温热</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>copperInsightMin=2;memoryMin=8</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>copperInsight=2;fragments=1;virtue=3</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>你把铜锈翻到背面，没有急着让任何人解释。
+背面没有完整的铜门，只留下许多手掌磨过的浅痕：有人在推门，有人在关门，也有人只是把掌心按在冷风里，替身后的人挡住第一道光。铜锈很快冷下去，只剩断口处一点温热。</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>6</v>
+      </c>
+      <c r="B142" t="n">
+        <v>82</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>把铜锈和几样旧物分开摆放</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>copperInsightMin=4;fragmentsMin=3</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>copperInsight=1;memory=1;virtue=4</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>铜锈、白羽、旧令、剑穗、药账和军册缺页被你分开放在地上。
+几样旧物互不相连，只有铜锈在你提到撤民、病榻和北墙灯时微微发热。它不像在认门，更像在认那些被门风逼到石阶下的人。</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>7</v>
+      </c>
+      <c r="B143" t="n">
+        <v>81</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>把铜锈留在门风照不到的地方</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>rustWitnessEnding</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>copperInsightMin=5;memoryMin=15;fragmentsMin=4;virtueMin=60</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>memory=3;fragments=1;virtue=8</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>你没有把铜锈贴上门缝。
+你把它放到门风照不到的石阶上。绿锈贴着石面慢慢冷下去，断口朝外，像一枚从门上剥落、又被许多人带回来的旧痂。</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>2</v>
+      </c>
+      <c r="B144" t="n">
+        <v>32</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>守在静息房外听潮声</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>path=冰心堂;iceLedgerMin=2</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>iceLedger=2;virtue=8;karma=-2;qingshiBond=1;years=-1</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>静息房里没有哭声，只有细得几乎听不见的呼吸。药庐少年还没有告诉你名字，只把一枚空药签递来，让你记下每一次停顿。
+你守到后半夜，才发现窗缝里吹来的风带着海腥味。</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>3</v>
+      </c>
+      <c r="B145" t="n">
+        <v>16</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>把带海腥味的脉案另放一格</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>path=冰心堂;iceLedgerMin=3</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>iceLedger=2;memory=1;qingshiBond=1;virtue=6</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>你把几页脉案分开：药味相同，病人的沉默却不同。有的人是疼到说不出话，有的人像被远处潮声带走了声音。
+药庐少年看见你的分法，第一次没有纠正，只把灯挪近了一点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>4</v>
+      </c>
+      <c r="B146" t="n">
+        <v>18</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>把药箱送到队尾</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>path=冰心堂;iceLedgerMin=4</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>iceLedger=1;virtue=8;karma=-2;qingshiBond=1;years=-1</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>队伍最末的人走得最慢，药箱却总被催着往前送。你和药庐少年把箱子抬回队尾，先给那个咳不出声的人换了温水。
+药庐少年没有谈铜门。他只说，冰心堂若听不见最轻的气息，就不配谈救天下。</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>5</v>
+      </c>
+      <c r="B147" t="n">
+        <v>12</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>请药庐少年先说海潮病人的脉案</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>path=冰心堂;iceLedgerMin=5;qingshiBondMin=3</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>iceLedger=2;virtue=8;karma=-2;qingshiBond=1;fragments=1;knownName=qingshi</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>药庐后堂没有人敢先说真相。药庐少年把海潮病人的脉案放到灯下，一页页翻给堂中长辈看。
+药庐少年：我叫清时。我不问谁该受罚，只问为什么这些人还没死，名字就已经被划掉了。</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>6</v>
+      </c>
+      <c r="B148" t="n">
+        <v>7</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>陪清时把海寂脉案封进药箱</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>afterBreak</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>path=冰心堂;knownName=qingshi;iceLedgerMin=6;qingshiBondMin=4</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>iceLedger=2;virtue=10;karma=-3;qingshiBond=2;fragments=1;years=-1</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>清时没有把海寂说成天灾，也没有把它推给某个仇人。他只是把脉案、药签和病人的名字一页页封进药箱。
+清时：若下一世还能遇见，请先听他们的呼吸。答案可以慢一点，人不能。</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>7</v>
+      </c>
+      <c r="B149" t="n">
+        <v>13</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>陪清时把药灯留给海风里的人</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>qingshiEnding</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>path=冰心堂;knownName=qingshi;iceLedgerMin=8;qingshiBondMin=5;virtueMin=70</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>virtue=14;memory=2;fragments=1</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>铜门前的风带着海腥味。清时没有向门后求答案，只把药灯一盏盏摆到病人身边。你陪他守到天亮，终于听见最轻的那口气续了回来。</t>
         </is>
       </c>
     </row>
@@ -4530,7 +5989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4738,7 +6197,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>冰心医毒线；药账、魂灯、寒毒，强调毒也可救人，药也可害人。</t>
+          <t>冰心堂年轻弟子。前期称药庐少年/药童，水镜前自报清时。核心不是揭穿阴谋，而是坚持先救仍有一口气的人。</t>
         </is>
       </c>
     </row>
@@ -4875,6 +6334,40 @@
       <c r="C20" t="inlineStr">
         <is>
           <t>玩家可以不拜任何门派，成为山海游侠或诸门客卿，通过替各门派和凡人送信、作证、救人来推进主线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>清时</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>海寂支线</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>以海潮病/海寂脉案承接东海与江南水患气质：潮声压住病人呼吸，药签、冷针、药账逐步拼出有人提前放弃病人的事实。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>冰心堂</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>门派脉络</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>冰心堂支线不让玩家越级决策。玩家先做药庐杂役、送药、记脉、护药箱，轮回加深后才凭亲眼见过的脉案影响水镜前的判断。</t>
         </is>
       </c>
     </row>
@@ -4889,7 +6382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D65"/>
+  <dimension ref="A1:D87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5065,12 +6558,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>assets/sect-new-pact.webp</t>
+          <t>assets/ferry-dawn-crowd.webp</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>门派选择、会盟余波</t>
+          <t>?????????????</t>
         </is>
       </c>
     </row>
@@ -6191,6 +7684,1084 @@
       <c r="D65" t="inlineStr">
         <is>
           <t>雪线交灯</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>afterBreak:6</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>1</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>assets/companions-pact.webp</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>同行之约新背景</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>afterBreak:7</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>assets/bronze-gate-v2.webp</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>铜门终局</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>afterBreak:7</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>2</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>assets/copper-gate.webp</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>铜门终局备选</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>afterBreak:7</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>3</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>assets/true-ascend.webp</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>天光终局备选</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>xuanhuiEnding</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>assets/xuanhui-snow-lamp.webp</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>玄晖雪灯结局背景</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>mofeiyunEnding</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>1</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>assets/mofeiyun-tide-mirror.webp</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>莫非云东海水镜结局背景</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>qingyangEnding</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>1</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>assets/qingyang-route.webp</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>青阳雨路结局背景</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>afterBreak:2</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>41</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>assets/tianji-north-wall-command.webp</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>天机营北墙、巡灯、竹筒军令</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>afterBreak:6</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>42</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>assets/tianji-shangxie-registry.webp</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>天机营水镜、上邪残页、军册</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>qiyeEnding</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>1</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>assets/qiye-shuofang-retreat.webp</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>朔方雪原、黄泉水、退路灯火</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>changqinEnding</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>1</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>assets/changqin-fire-temple.webp</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>太子长琴线、熔岩旧殿、无人物场景</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>xuanhuiEnding</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>2</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>assets/xuanhui-snow-lantern-dawn.webp</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>???????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>mofeiyunEnding</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>2</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>assets/mofeiyun-star-tide.webp</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>????????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>qingyangEnding</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>2</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>assets/qingyang-side-gate.webp</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>???????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>qiyeEnding</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>2</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>assets/qiye-north-wall-dawn.webp</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>???????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>changqinEnding</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>2</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>assets/changqin-ember-zither.webp</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>?????????????</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>qingshiEnding</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>1</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>assets/medicine-ledger-night.webp</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>清时结局、药灯、海寂脉案</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>qingshiEnding</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>2</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>assets/iceheart-hall.webp</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>冰心堂、药灯、救人</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>afterBreak:2</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>90</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>assets/iceheart-rain-medicine-hut.webp</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>冰心堂雨夜药庐、海潮病、清时前期</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>afterBreak:4</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>91</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>assets/iceheart-snow-medicine-chest.webp</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>冰心堂雪线药箱、队尾救治</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>qingshiEnding</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>3</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>assets/qingshi-medicine-lantern-dawn.webp</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>清时结局、海风药灯、药账天明</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>medicineEnding</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>90</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>assets/qingshi-medicine-lantern-dawn.webp</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>冰心堂结局备选、药灯天明</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Aliases</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>PortraitClass</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Tone</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>旁白</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>旁白|叙述</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>narrator</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>hidden</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>neutral</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>场景叙述，不显示立绘。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>你</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>你|玩家|自己</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>player</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>玩家对白或内心回应。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>tianji_guard</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>天机营校尉</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>天机营校尉|校尉|守门校尉|巡夜人</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>tianji</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>iron</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>天机营秩序线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ice_boy</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>药庐少年</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>药庐少年|药童|童子|冰心堂弟子|清时</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>ice</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>medicine</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>清时线。前期只能称药庐少年/药童；水镜前自报后才可称清时。头像只用于冰心堂药庐、药账、海寂脉案相关对白。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>sword_guest</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>雨亭剑客</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>雨亭剑客|剑客|青阳|青阳少昊</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>sword</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>rain</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>弈剑线，后续接青阳少昊。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>star_watcher</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>观星者</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>观星者|观星的人|莫非云|云麓弟子</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>star</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>star</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>云麓线，后续接莫非云。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>mirror_shadow</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>镜中影</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>镜中影|影子|镜室里的人</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>mirror</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>mirror</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>太虚线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>shadow_blade</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>递牌人</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>递牌人|持刀的人|夜哭|旧巷人</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>shadow</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>shadow</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>魍魉线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>feather_mechanic</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>机关师</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>机关师|遗墨|翎羽弟子</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>feather</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>wood</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>翎羽线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>fire_woman</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>炉边女子</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>炉边女子|荒火弟子|搬炭的人</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>fire</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>fire</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>荒火线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ferry_scholar</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>车辕书生</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>车辕上的书生|书生|渡口行人</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>scholar</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>wanderer</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>游侠/渡口线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>old_boatman</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>老船夫</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>老船夫|船夫</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>boatman</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>water</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>城内杂役与渡口线。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>lamp_keeper</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>点灯人</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>点灯人|雪灯人|玄晖|东皇太一</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>lamp</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>sun</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>玄晖/金乌主轴。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>孩子</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>孩子|小孩</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>soft</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>被救助者或城外人。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>changqin_echo</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>火中琴声</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>火中琴声|琴声|太子长琴|长琴</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>fire</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>qiye_commander</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>朔方城主</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>朔方城主|七夜|幽都统帅|武观</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>iron</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>right</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>cold</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>天机营遭遇的外部压力：七夜/武观，只在朔方旧卷与上邪残页后逐步揭示。</t>
         </is>
       </c>
     </row>

</xml_diff>